<commit_message>
added freq_thres_h and question
</commit_message>
<xml_diff>
--- a/Distributions.xlsx
+++ b/Distributions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aaltofi-my.sharepoint.com/personal/samuel_salin_aalto_fi/Documents/Desktop/Risk Elicitation/RE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_BBF9AF74AC20D3FF2286BA73C3D10CC99D880FBC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B475AB59-9C80-4B51-ABA7-F0F6F2694E65}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="11_BA4D2FB74CA8045DC74C1AC6005315D59D888FE4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E53CF80-D76A-45FC-B8D4-F6B92E7F8969}"/>
   <bookViews>
     <workbookView xWindow="-5160" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="29">
   <si>
     <t>D1</t>
   </si>
@@ -109,9 +109,6 @@
     <t>Variation 2.2: Random allocation of outcomes to situations by state (e.g., same-row observations in column B and column C form an outcome pair that cannot be broken up, so that the structure of dependence is fixed)</t>
   </si>
   <si>
-    <t>Round Thresholds: FREQ_THRES_L / TAIL_THRES_L / TAIL_THRES_H per distribution (same threshold used for both alternatives in a round that draws this distribution; edit the numbers below directly - no code changes needed)</t>
-  </si>
-  <si>
     <t>FREQ_THRES_L</t>
   </si>
   <si>
@@ -119,6 +116,12 @@
   </si>
   <si>
     <t>TAIL_THRES_H</t>
+  </si>
+  <si>
+    <t>FREQ_THRES_H</t>
+  </si>
+  <si>
+    <t>Round Thresholds: FREQ_THRES_L /H and  TAIL_THRES_L / H per distribution (same threshold used for both alternatives in a round that draws this distribution; edit the numbers below directly - no code changes needed)</t>
   </si>
 </sst>
 </file>
@@ -540,7 +543,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:AB109"/>
+  <dimension ref="A2:AB110"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="198.81640625" bestFit="1" customWidth="1"/>
@@ -2061,27 +2064,27 @@
       </c>
       <c r="C29" s="1">
         <f t="array" aca="1" ref="C29:C39" ca="1">_xlfn.SORTBY(C3:C13,_xlfn.RANDARRAY(ROWS(C3:C13)))</f>
-        <v>0.6</v>
+        <v>0.79999999999999993</v>
       </c>
       <c r="D29" s="1">
         <f t="array" aca="1" ref="D29:D39" ca="1">_xlfn.SORTBY(D3:D13,_xlfn.RANDARRAY(ROWS(D3:D13)))</f>
-        <v>0</v>
+        <v>0.79999999999999982</v>
       </c>
       <c r="E29" s="1">
         <f t="array" aca="1" ref="E29:E39" ca="1">_xlfn.SORTBY(E3:E13,_xlfn.RANDARRAY(ROWS(E3:E13)))</f>
-        <v>-0.20000000000000009</v>
+        <v>9.9999999999999867E-2</v>
       </c>
       <c r="F29" s="1">
         <f t="array" aca="1" ref="F29:F39" ca="1">_xlfn.SORTBY(F3:F13,_xlfn.RANDARRAY(ROWS(F3:F13)))</f>
-        <v>-0.20000000000000021</v>
+        <v>-2</v>
       </c>
       <c r="G29" s="1">
         <f t="array" aca="1" ref="G29:G39" ca="1">_xlfn.SORTBY(G3:G13,_xlfn.RANDARRAY(ROWS(G3:G13)))</f>
-        <v>-1.1000000000000001</v>
+        <v>-0.59999999999999987</v>
       </c>
       <c r="H29" s="1">
         <f t="array" aca="1" ref="H29:H39" ca="1">_xlfn.SORTBY(H3:H13,_xlfn.RANDARRAY(ROWS(H3:H13)))</f>
-        <v>1.9</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="I29" s="1">
         <f t="array" aca="1" ref="I29:I39" ca="1">_xlfn.SORTBY(I3:I13,_xlfn.RANDARRAY(ROWS(I3:I13)))</f>
@@ -2089,51 +2092,51 @@
       </c>
       <c r="J29" s="1">
         <f t="array" aca="1" ref="J29:J39" ca="1">_xlfn.SORTBY(J3:J13,_xlfn.RANDARRAY(ROWS(J3:J13)))</f>
-        <v>-0.70000000000000007</v>
+        <v>-1.9</v>
       </c>
       <c r="K29" s="1">
         <f t="array" aca="1" ref="K29:K39" ca="1">_xlfn.SORTBY(K3:K13,_xlfn.RANDARRAY(ROWS(K3:K13)))</f>
-        <v>-1</v>
+        <v>-0.59999999999999976</v>
       </c>
       <c r="L29" s="1">
         <f t="array" aca="1" ref="L29:L39" ca="1">_xlfn.SORTBY(L3:L13,_xlfn.RANDARRAY(ROWS(L3:L13)))</f>
-        <v>2</v>
+        <v>0.89</v>
       </c>
       <c r="M29" s="1">
         <f t="array" aca="1" ref="M29:M39" ca="1">_xlfn.SORTBY(M3:M13,_xlfn.RANDARRAY(ROWS(M3:M13)))</f>
-        <v>1.1499999999999999</v>
+        <v>1.07</v>
       </c>
       <c r="N29" s="1">
         <f t="array" aca="1" ref="N29:N39" ca="1">_xlfn.SORTBY(N3:N13,_xlfn.RANDARRAY(ROWS(N3:N13)))</f>
-        <v>-0.12</v>
+        <v>1</v>
       </c>
       <c r="O29" s="1">
         <f t="array" aca="1" ref="O29:O39" ca="1">_xlfn.SORTBY(O3:O13,_xlfn.RANDARRAY(ROWS(O3:O13)))</f>
-        <v>0.15000000000000011</v>
+        <v>0.12000000000000011</v>
       </c>
       <c r="P29" s="1">
         <f t="array" aca="1" ref="P29:P39" ca="1">_xlfn.SORTBY(P3:P13,_xlfn.RANDARRAY(ROWS(P3:P13)))</f>
-        <v>-1.08</v>
+        <v>-1.05</v>
       </c>
       <c r="Q29" s="1">
         <f t="array" aca="1" ref="Q29:Q39" ca="1">_xlfn.SORTBY(Q3:Q13,_xlfn.RANDARRAY(ROWS(Q3:Q13)))</f>
-        <v>-2</v>
+        <v>-0.94</v>
       </c>
       <c r="R29" s="1">
         <f t="array" aca="1" ref="R29:R39" ca="1">_xlfn.SORTBY(R3:R13,_xlfn.RANDARRAY(ROWS(R3:R13)))</f>
-        <v>2.1</v>
+        <v>0.95</v>
       </c>
       <c r="S29" s="1">
         <f t="array" aca="1" ref="S29:S39" ca="1">_xlfn.SORTBY(S3:S13,_xlfn.RANDARRAY(ROWS(S3:S13)))</f>
-        <v>1.1599999999999999</v>
+        <v>1.23</v>
       </c>
       <c r="T29" s="1">
         <f t="array" aca="1" ref="T29:T39" ca="1">_xlfn.SORTBY(T3:T13,_xlfn.RANDARRAY(ROWS(T3:T13)))</f>
-        <v>-0.1</v>
+        <v>-1.1599999999999999</v>
       </c>
       <c r="U29" s="1">
         <f t="array" aca="1" ref="U29:U39" ca="1">_xlfn.SORTBY(U3:U13,_xlfn.RANDARRAY(ROWS(U3:U13)))</f>
-        <v>-0.95999999999999985</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.35">
@@ -2142,83 +2145,83 @@
       </c>
       <c r="B30" s="1">
         <f ca="1"/>
+        <v>2</v>
+      </c>
+      <c r="C30" s="1">
+        <f ca="1"/>
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D30" s="1">
+        <f ca="1"/>
+        <v>-0.2</v>
+      </c>
+      <c r="E30" s="1">
+        <f ca="1"/>
+        <v>0.40000000000000008</v>
+      </c>
+      <c r="F30" s="1">
+        <f ca="1"/>
+        <v>-1</v>
+      </c>
+      <c r="G30" s="1">
+        <f ca="1"/>
+        <v>-0.8</v>
+      </c>
+      <c r="H30" s="1">
+        <f ca="1"/>
+        <v>0.5</v>
+      </c>
+      <c r="I30" s="1">
+        <f ca="1"/>
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="J30" s="1">
+        <f ca="1"/>
+        <v>-0.70000000000000007</v>
+      </c>
+      <c r="K30" s="1">
+        <f ca="1"/>
+        <v>-1.5</v>
+      </c>
+      <c r="L30" s="1">
+        <f ca="1"/>
+        <v>0.85</v>
+      </c>
+      <c r="M30" s="1">
+        <f ca="1"/>
+        <v>1.08</v>
+      </c>
+      <c r="N30" s="1">
+        <f ca="1"/>
+        <v>-0.12</v>
+      </c>
+      <c r="O30" s="1">
+        <f ca="1"/>
+        <v>5.0000000000000037E-2</v>
+      </c>
+      <c r="P30" s="1">
+        <f ca="1"/>
         <v>0</v>
       </c>
-      <c r="C30" s="1">
-        <f ca="1"/>
-        <v>1.2</v>
-      </c>
-      <c r="D30" s="1">
-        <f ca="1"/>
-        <v>0.2</v>
-      </c>
-      <c r="E30" s="1">
-        <f ca="1"/>
-        <v>-0.4</v>
-      </c>
-      <c r="F30" s="1">
-        <f ca="1"/>
-        <v>-1.4</v>
-      </c>
-      <c r="G30" s="1">
-        <f ca="1"/>
-        <v>-0.8</v>
-      </c>
-      <c r="H30" s="1">
-        <f ca="1"/>
-        <v>0.5</v>
-      </c>
-      <c r="I30" s="1">
-        <f ca="1"/>
-        <v>1.4</v>
-      </c>
-      <c r="J30" s="1">
-        <f ca="1"/>
-        <v>-1.1000000000000001</v>
-      </c>
-      <c r="K30" s="1">
-        <f ca="1"/>
-        <v>-0.9</v>
-      </c>
-      <c r="L30" s="1">
-        <f ca="1"/>
-        <v>0.86</v>
-      </c>
-      <c r="M30" s="1">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="N30" s="1">
-        <f ca="1"/>
-        <v>-0.14000000000000001</v>
-      </c>
-      <c r="O30" s="1">
-        <f ca="1"/>
-        <v>6.0000000000000053E-2</v>
-      </c>
-      <c r="P30" s="1">
-        <f ca="1"/>
-        <v>-1.06</v>
-      </c>
       <c r="Q30" s="1">
         <f ca="1"/>
-        <v>-0.94</v>
+        <v>-0.84999999999999987</v>
       </c>
       <c r="R30" s="1">
         <f ca="1"/>
-        <v>0.98</v>
+        <v>1.01</v>
       </c>
       <c r="S30" s="1">
         <f ca="1"/>
-        <v>1.22</v>
+        <v>0.1</v>
       </c>
       <c r="T30" s="1">
         <f ca="1"/>
-        <v>-1.1499999999999999</v>
+        <v>-1.25</v>
       </c>
       <c r="U30" s="1">
         <f ca="1"/>
-        <v>-1.05</v>
+        <v>-0.96999999999999986</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.35">
@@ -2227,7 +2230,7 @@
       </c>
       <c r="B31" s="1">
         <f ca="1"/>
-        <v>1.4</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="C31" s="1">
         <f ca="1"/>
@@ -2235,75 +2238,75 @@
       </c>
       <c r="D31" s="1">
         <f ca="1"/>
-        <v>0.59999999999999987</v>
+        <v>-1</v>
       </c>
       <c r="E31" s="1">
         <f ca="1"/>
-        <v>-0.1000000000000001</v>
+        <v>-0.20000000000000009</v>
       </c>
       <c r="F31" s="1">
         <f ca="1"/>
-        <v>-1</v>
+        <v>-0.60000000000000009</v>
       </c>
       <c r="G31" s="1">
         <f ca="1"/>
-        <v>-1.3</v>
+        <v>-1.2</v>
       </c>
       <c r="H31" s="1">
         <f ca="1"/>
+        <v>1.5</v>
+      </c>
+      <c r="I31" s="1">
+        <f ca="1"/>
+        <v>1.2</v>
+      </c>
+      <c r="J31" s="1">
+        <f ca="1"/>
+        <v>-0.50000000000000011</v>
+      </c>
+      <c r="K31" s="1">
+        <f ca="1"/>
+        <v>-0.79999999999999993</v>
+      </c>
+      <c r="L31" s="1">
+        <f ca="1"/>
+        <v>0.88</v>
+      </c>
+      <c r="M31" s="1">
+        <f ca="1"/>
+        <v>1.1399999999999999</v>
+      </c>
+      <c r="N31" s="1">
+        <f ca="1"/>
+        <v>-0.15</v>
+      </c>
+      <c r="O31" s="1">
+        <f ca="1"/>
+        <v>0.1400000000000001</v>
+      </c>
+      <c r="P31" s="1">
+        <f ca="1"/>
+        <v>-1.1499999999999999</v>
+      </c>
+      <c r="Q31" s="1">
+        <f ca="1"/>
+        <v>-0.87999999999999989</v>
+      </c>
+      <c r="R31" s="1">
+        <f ca="1"/>
         <v>2.1</v>
       </c>
-      <c r="I31" s="1">
-        <f ca="1"/>
-        <v>1.2</v>
-      </c>
-      <c r="J31" s="1">
-        <f ca="1"/>
-        <v>-1.3</v>
-      </c>
-      <c r="K31" s="1">
-        <f ca="1"/>
-        <v>-1.1000000000000001</v>
-      </c>
-      <c r="L31" s="1">
-        <f ca="1"/>
-        <v>0.92</v>
-      </c>
-      <c r="M31" s="1">
-        <f ca="1"/>
-        <v>1.1399999999999999</v>
-      </c>
-      <c r="N31" s="1">
-        <f ca="1"/>
-        <v>-0.11</v>
-      </c>
-      <c r="O31" s="1">
-        <f ca="1"/>
-        <v>8.0000000000000071E-2</v>
-      </c>
-      <c r="P31" s="1">
-        <f ca="1"/>
-        <v>-1.05</v>
-      </c>
-      <c r="Q31" s="1">
-        <f ca="1"/>
-        <v>-0.87999999999999989</v>
-      </c>
-      <c r="R31" s="1">
-        <f ca="1"/>
-        <v>1.01</v>
-      </c>
       <c r="S31" s="1">
         <f ca="1"/>
-        <v>1.1499999999999999</v>
+        <v>1.24</v>
       </c>
       <c r="T31" s="1">
         <f ca="1"/>
-        <v>-1.19</v>
+        <v>-1.22</v>
       </c>
       <c r="U31" s="1">
         <f ca="1"/>
-        <v>-2.1</v>
+        <v>-0.95999999999999985</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.35">
@@ -2312,23 +2315,23 @@
       </c>
       <c r="B32" s="1">
         <f ca="1"/>
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="C32" s="1">
         <f ca="1"/>
-        <v>0.89999999999999991</v>
+        <v>0.99999999999999989</v>
       </c>
       <c r="D32" s="1">
         <f ca="1"/>
-        <v>0.99999999999999978</v>
+        <v>-0.6</v>
       </c>
       <c r="E32" s="1">
         <f ca="1"/>
-        <v>9.9999999999999867E-2</v>
+        <v>0</v>
       </c>
       <c r="F32" s="1">
         <f ca="1"/>
-        <v>0</v>
+        <v>-1.4</v>
       </c>
       <c r="G32" s="1">
         <f ca="1"/>
@@ -2336,59 +2339,59 @@
       </c>
       <c r="H32" s="1">
         <f ca="1"/>
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="I32" s="1">
         <f ca="1"/>
-        <v>0.7</v>
+        <v>0.99999999999999989</v>
       </c>
       <c r="J32" s="1">
         <f ca="1"/>
-        <v>-0.9</v>
+        <v>-1.3</v>
       </c>
       <c r="K32" s="1">
         <f ca="1"/>
-        <v>-1.6</v>
+        <v>-1.3</v>
       </c>
       <c r="L32" s="1">
         <f ca="1"/>
-        <v>0.94000000000000006</v>
+        <v>0.92</v>
       </c>
       <c r="M32" s="1">
         <f ca="1"/>
-        <v>1.07</v>
+        <v>1.05</v>
       </c>
       <c r="N32" s="1">
         <f ca="1"/>
-        <v>-7.999999999999996E-2</v>
+        <v>-4.9999999999999933E-2</v>
       </c>
       <c r="O32" s="1">
         <f ca="1"/>
-        <v>0.13000000000000009</v>
+        <v>7.0000000000000062E-2</v>
       </c>
       <c r="P32" s="1">
         <f ca="1"/>
-        <v>-1.1100000000000001</v>
+        <v>-1.06</v>
       </c>
       <c r="Q32" s="1">
         <f ca="1"/>
-        <v>-0.90999999999999992</v>
+        <v>-0.95</v>
       </c>
       <c r="R32" s="1">
         <f ca="1"/>
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="S32" s="1">
         <f ca="1"/>
-        <v>1.25</v>
+        <v>1.21</v>
       </c>
       <c r="T32" s="1">
         <f ca="1"/>
-        <v>-1.21</v>
+        <v>-1.24</v>
       </c>
       <c r="U32" s="1">
         <f ca="1"/>
-        <v>-1.02</v>
+        <v>-1.03</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.35">
@@ -2397,47 +2400,47 @@
       </c>
       <c r="B33" s="1">
         <f ca="1"/>
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="C33" s="1">
         <f ca="1"/>
-        <v>1.3</v>
+        <v>0.89999999999999991</v>
       </c>
       <c r="D33" s="1">
         <f ca="1"/>
-        <v>0.79999999999999982</v>
+        <v>-0.8</v>
       </c>
       <c r="E33" s="1">
         <f ca="1"/>
-        <v>-0.5</v>
+        <v>-0.1000000000000001</v>
       </c>
       <c r="F33" s="1">
         <f ca="1"/>
-        <v>-0.40000000000000008</v>
+        <v>-0.20000000000000021</v>
       </c>
       <c r="G33" s="1">
         <f ca="1"/>
-        <v>-1.4</v>
+        <v>-0.7</v>
       </c>
       <c r="H33" s="1">
         <f ca="1"/>
-        <v>0.70000000000000007</v>
+        <v>1.9</v>
       </c>
       <c r="I33" s="1">
         <f ca="1"/>
-        <v>0.6</v>
+        <v>1.4</v>
       </c>
       <c r="J33" s="1">
         <f ca="1"/>
-        <v>-1.5</v>
+        <v>-2.1</v>
       </c>
       <c r="K33" s="1">
         <f ca="1"/>
-        <v>-0.79999999999999993</v>
+        <v>-1</v>
       </c>
       <c r="L33" s="1">
         <f ca="1"/>
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="M33" s="1">
         <f ca="1"/>
@@ -2445,35 +2448,35 @@
       </c>
       <c r="N33" s="1">
         <f ca="1"/>
-        <v>-0.13</v>
+        <v>-0.11</v>
       </c>
       <c r="O33" s="1">
         <f ca="1"/>
-        <v>0.12000000000000011</v>
+        <v>8.0000000000000071E-2</v>
       </c>
       <c r="P33" s="1">
         <f ca="1"/>
-        <v>-1.1200000000000001</v>
+        <v>-1.1299999999999999</v>
       </c>
       <c r="Q33" s="1">
         <f ca="1"/>
-        <v>-0.86999999999999988</v>
+        <v>-0.8899999999999999</v>
       </c>
       <c r="R33" s="1">
         <f ca="1"/>
-        <v>0.95</v>
+        <v>1.03</v>
       </c>
       <c r="S33" s="1">
         <f ca="1"/>
-        <v>1.18</v>
+        <v>1.25</v>
       </c>
       <c r="T33" s="1">
         <f ca="1"/>
-        <v>-1.25</v>
+        <v>-1.23</v>
       </c>
       <c r="U33" s="1">
         <f ca="1"/>
-        <v>-1.01</v>
+        <v>-1.05</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.35">
@@ -2482,39 +2485,39 @@
       </c>
       <c r="B34" s="1">
         <f ca="1"/>
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="C34" s="1">
         <f ca="1"/>
-        <v>1.1000000000000001</v>
+        <v>1.3</v>
       </c>
       <c r="D34" s="1">
         <f ca="1"/>
-        <v>-0.39999999999999991</v>
+        <v>0.2</v>
       </c>
       <c r="E34" s="1">
         <f ca="1"/>
-        <v>0.40000000000000008</v>
+        <v>0.3</v>
       </c>
       <c r="F34" s="1">
         <f ca="1"/>
-        <v>-1.2</v>
+        <v>-1.6</v>
       </c>
       <c r="G34" s="1">
         <f ca="1"/>
-        <v>-0.7</v>
+        <v>-1.4</v>
       </c>
       <c r="H34" s="1">
         <f ca="1"/>
-        <v>1.1000000000000001</v>
+        <v>0.70000000000000007</v>
       </c>
       <c r="I34" s="1">
         <f ca="1"/>
-        <v>1.5</v>
+        <v>0.6</v>
       </c>
       <c r="J34" s="1">
         <f ca="1"/>
-        <v>-1.9</v>
+        <v>-1.5</v>
       </c>
       <c r="K34" s="1">
         <f ca="1"/>
@@ -2522,43 +2525,43 @@
       </c>
       <c r="L34" s="1">
         <f ca="1"/>
-        <v>0.93</v>
+        <v>0.95000000000000007</v>
       </c>
       <c r="M34" s="1">
         <f ca="1"/>
-        <v>1.06</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="N34" s="1">
         <f ca="1"/>
-        <v>-4.9999999999999933E-2</v>
+        <v>-0.13</v>
       </c>
       <c r="O34" s="1">
         <f ca="1"/>
-        <v>0.1400000000000001</v>
+        <v>9.000000000000008E-2</v>
       </c>
       <c r="P34" s="1">
         <f ca="1"/>
-        <v>-1.0900000000000001</v>
+        <v>-1.1200000000000001</v>
       </c>
       <c r="Q34" s="1">
         <f ca="1"/>
-        <v>-0.8899999999999999</v>
+        <v>-0.85999999999999988</v>
       </c>
       <c r="R34" s="1">
         <f ca="1"/>
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="S34" s="1">
         <f ca="1"/>
-        <v>1.23</v>
+        <v>1.18</v>
       </c>
       <c r="T34" s="1">
         <f ca="1"/>
-        <v>-1.24</v>
+        <v>-1.21</v>
       </c>
       <c r="U34" s="1">
         <f ca="1"/>
-        <v>-0.97999999999999987</v>
+        <v>-1.01</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.35">
@@ -2567,15 +2570,15 @@
       </c>
       <c r="B35" s="1">
         <f ca="1"/>
-        <v>0.60000000000000009</v>
+        <v>0.2</v>
       </c>
       <c r="C35" s="1">
         <f ca="1"/>
-        <v>0.79999999999999993</v>
+        <v>1.2</v>
       </c>
       <c r="D35" s="1">
         <f ca="1"/>
-        <v>0.39999999999999991</v>
+        <v>0</v>
       </c>
       <c r="E35" s="1">
         <f ca="1"/>
@@ -2583,11 +2586,11 @@
       </c>
       <c r="F35" s="1">
         <f ca="1"/>
-        <v>-1.8</v>
+        <v>-0.8</v>
       </c>
       <c r="G35" s="1">
         <f ca="1"/>
-        <v>-1.5</v>
+        <v>-1.3</v>
       </c>
       <c r="H35" s="1">
         <f ca="1"/>
@@ -2599,27 +2602,27 @@
       </c>
       <c r="J35" s="1">
         <f ca="1"/>
-        <v>-2.1</v>
+        <v>-0.30000000000000021</v>
       </c>
       <c r="K35" s="1">
         <f ca="1"/>
-        <v>-1.3</v>
+        <v>-0.69999999999999984</v>
       </c>
       <c r="L35" s="1">
         <f ca="1"/>
-        <v>0.87</v>
+        <v>0.94000000000000006</v>
       </c>
       <c r="M35" s="1">
         <f ca="1"/>
-        <v>1.0900000000000001</v>
+        <v>1.1200000000000001</v>
       </c>
       <c r="N35" s="1">
         <f ca="1"/>
-        <v>-0.15</v>
+        <v>-6.9999999999999951E-2</v>
       </c>
       <c r="O35" s="1">
         <f ca="1"/>
-        <v>9.000000000000008E-2</v>
+        <v>6.0000000000000053E-2</v>
       </c>
       <c r="P35" s="1">
         <f ca="1"/>
@@ -2627,7 +2630,7 @@
       </c>
       <c r="Q35" s="1">
         <f ca="1"/>
-        <v>-0.91999999999999993</v>
+        <v>-0.86999999999999988</v>
       </c>
       <c r="R35" s="1">
         <f ca="1"/>
@@ -2639,11 +2642,11 @@
       </c>
       <c r="T35" s="1">
         <f ca="1"/>
-        <v>-1.18</v>
+        <v>-1.17</v>
       </c>
       <c r="U35" s="1">
         <f ca="1"/>
-        <v>-0.98999999999999988</v>
+        <v>-0.94999999999999984</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.35">
@@ -2652,79 +2655,79 @@
       </c>
       <c r="B36" s="1">
         <f ca="1"/>
-        <v>0.2</v>
+        <v>1.6</v>
       </c>
       <c r="C36" s="1">
         <f ca="1"/>
-        <v>0.99999999999999989</v>
+        <v>1.4</v>
       </c>
       <c r="D36" s="1">
         <f ca="1"/>
-        <v>-0.8</v>
+        <v>-0.39999999999999991</v>
       </c>
       <c r="E36" s="1">
         <f ca="1"/>
-        <v>-0.3</v>
+        <v>0.50000000000000022</v>
       </c>
       <c r="F36" s="1">
         <f ca="1"/>
-        <v>-2</v>
+        <v>-0.40000000000000008</v>
       </c>
       <c r="G36" s="1">
         <f ca="1"/>
-        <v>-0.49999999999999978</v>
+        <v>-1.1000000000000001</v>
       </c>
       <c r="H36" s="1">
         <f ca="1"/>
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
       <c r="I36" s="1">
         <f ca="1"/>
-        <v>0.99999999999999989</v>
+        <v>0.89999999999999991</v>
       </c>
       <c r="J36" s="1">
         <f ca="1"/>
-        <v>-0.50000000000000011</v>
+        <v>-0.9</v>
       </c>
       <c r="K36" s="1">
         <f ca="1"/>
-        <v>-0.59999999999999976</v>
+        <v>-1.1000000000000001</v>
       </c>
       <c r="L36" s="1">
         <f ca="1"/>
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="M36" s="1">
         <f ca="1"/>
-        <v>1.1100000000000001</v>
+        <v>1.06</v>
       </c>
       <c r="N36" s="1">
         <f ca="1"/>
-        <v>-6.9999999999999951E-2</v>
+        <v>-8.9999999999999969E-2</v>
       </c>
       <c r="O36" s="1">
         <f ca="1"/>
-        <v>5.0000000000000037E-2</v>
+        <v>-1</v>
       </c>
       <c r="P36" s="1">
         <f ca="1"/>
-        <v>-1.1299999999999999</v>
+        <v>-1.1100000000000001</v>
       </c>
       <c r="Q36" s="1">
         <f ca="1"/>
-        <v>-0.85999999999999988</v>
+        <v>-0.90999999999999992</v>
       </c>
       <c r="R36" s="1">
         <f ca="1"/>
-        <v>1.05</v>
+        <v>0.97</v>
       </c>
       <c r="S36" s="1">
         <f ca="1"/>
-        <v>1.24</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="T36" s="1">
         <f ca="1"/>
-        <v>-1.1599999999999999</v>
+        <v>-0.1</v>
       </c>
       <c r="U36" s="1">
         <f ca="1"/>
@@ -2737,7 +2740,7 @@
       </c>
       <c r="B37" s="1">
         <f ca="1"/>
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="C37" s="1">
         <f ca="1"/>
@@ -2745,75 +2748,75 @@
       </c>
       <c r="D37" s="1">
         <f ca="1"/>
+        <v>0.39999999999999991</v>
+      </c>
+      <c r="E37" s="1">
+        <f ca="1"/>
+        <v>-0.3</v>
+      </c>
+      <c r="F37" s="1">
+        <f ca="1"/>
+        <v>0</v>
+      </c>
+      <c r="G37" s="1">
+        <f ca="1"/>
         <v>-1</v>
       </c>
-      <c r="E37" s="1">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="F37" s="1">
-        <f ca="1"/>
-        <v>-0.8</v>
-      </c>
-      <c r="G37" s="1">
-        <f ca="1"/>
-        <v>-1.2</v>
-      </c>
       <c r="H37" s="1">
         <f ca="1"/>
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="I37" s="1">
         <f ca="1"/>
-        <v>0.89999999999999991</v>
+        <v>1.5</v>
       </c>
       <c r="J37" s="1">
         <f ca="1"/>
-        <v>-0.30000000000000021</v>
+        <v>-0.1</v>
       </c>
       <c r="K37" s="1">
         <f ca="1"/>
-        <v>-0.69999999999999984</v>
+        <v>-1.6</v>
       </c>
       <c r="L37" s="1">
         <f ca="1"/>
-        <v>0.95000000000000007</v>
+        <v>2</v>
       </c>
       <c r="M37" s="1">
         <f ca="1"/>
-        <v>1.1200000000000001</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="N37" s="1">
         <f ca="1"/>
-        <v>1</v>
+        <v>-0.14000000000000001</v>
       </c>
       <c r="O37" s="1">
         <f ca="1"/>
-        <v>0.1100000000000001</v>
+        <v>0.15000000000000011</v>
       </c>
       <c r="P37" s="1">
         <f ca="1"/>
-        <v>-1.1399999999999999</v>
+        <v>-1.08</v>
       </c>
       <c r="Q37" s="1">
         <f ca="1"/>
-        <v>-0.95</v>
+        <v>-2</v>
       </c>
       <c r="R37" s="1">
         <f ca="1"/>
-        <v>1.02</v>
+        <v>1.05</v>
       </c>
       <c r="S37" s="1">
         <f ca="1"/>
-        <v>1.19</v>
+        <v>1.1599999999999999</v>
       </c>
       <c r="T37" s="1">
         <f ca="1"/>
-        <v>-1.22</v>
+        <v>-1.18</v>
       </c>
       <c r="U37" s="1">
         <f ca="1"/>
-        <v>-0.96999999999999986</v>
+        <v>-0.98999999999999988</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.35">
@@ -2822,7 +2825,7 @@
       </c>
       <c r="B38" s="1">
         <f ca="1"/>
-        <v>0.4</v>
+        <v>1.4</v>
       </c>
       <c r="C38" s="1">
         <f ca="1"/>
@@ -2830,31 +2833,31 @@
       </c>
       <c r="D38" s="1">
         <f ca="1"/>
-        <v>-0.2</v>
+        <v>0.59999999999999987</v>
       </c>
       <c r="E38" s="1">
         <f ca="1"/>
-        <v>0.3</v>
+        <v>-0.5</v>
       </c>
       <c r="F38" s="1">
         <f ca="1"/>
-        <v>-0.60000000000000009</v>
+        <v>-1.8</v>
       </c>
       <c r="G38" s="1">
         <f ca="1"/>
-        <v>-1</v>
+        <v>-1.5</v>
       </c>
       <c r="H38" s="1">
         <f ca="1"/>
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="I38" s="1">
         <f ca="1"/>
-        <v>1.1000000000000001</v>
+        <v>0.7</v>
       </c>
       <c r="J38" s="1">
         <f ca="1"/>
-        <v>-0.1</v>
+        <v>-1.1000000000000001</v>
       </c>
       <c r="K38" s="1">
         <f ca="1"/>
@@ -2862,43 +2865,43 @@
       </c>
       <c r="L38" s="1">
         <f ca="1"/>
-        <v>0.88</v>
+        <v>0.93</v>
       </c>
       <c r="M38" s="1">
         <f ca="1"/>
-        <v>1.05</v>
+        <v>1.0900000000000001</v>
       </c>
       <c r="N38" s="1">
         <f ca="1"/>
-        <v>-5.9999999999999942E-2</v>
+        <v>-7.999999999999996E-2</v>
       </c>
       <c r="O38" s="1">
         <f ca="1"/>
-        <v>7.0000000000000062E-2</v>
+        <v>0.13000000000000009</v>
       </c>
       <c r="P38" s="1">
         <f ca="1"/>
+        <v>-1.0900000000000001</v>
+      </c>
+      <c r="Q38" s="1">
+        <f ca="1"/>
+        <v>-0.92999999999999994</v>
+      </c>
+      <c r="R38" s="1">
+        <f ca="1"/>
+        <v>1.02</v>
+      </c>
+      <c r="S38" s="1">
+        <f ca="1"/>
+        <v>1.22</v>
+      </c>
+      <c r="T38" s="1">
+        <f ca="1"/>
         <v>-1.1499999999999999</v>
       </c>
-      <c r="Q38" s="1">
-        <f ca="1"/>
-        <v>-0.92999999999999994</v>
-      </c>
-      <c r="R38" s="1">
-        <f ca="1"/>
-        <v>1.03</v>
-      </c>
-      <c r="S38" s="1">
-        <f ca="1"/>
-        <v>0.1</v>
-      </c>
-      <c r="T38" s="1">
-        <f ca="1"/>
-        <v>-1.17</v>
-      </c>
       <c r="U38" s="1">
         <f ca="1"/>
-        <v>-1.03</v>
+        <v>-1.02</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.35">
@@ -2907,31 +2910,31 @@
       </c>
       <c r="B39" s="1">
         <f ca="1"/>
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="C39" s="1">
         <f ca="1"/>
-        <v>1.4</v>
+        <v>0.6</v>
       </c>
       <c r="D39" s="1">
         <f ca="1"/>
-        <v>-0.6</v>
+        <v>0.99999999999999978</v>
       </c>
       <c r="E39" s="1">
         <f ca="1"/>
-        <v>0.50000000000000022</v>
+        <v>-0.4</v>
       </c>
       <c r="F39" s="1">
         <f ca="1"/>
-        <v>-1.6</v>
+        <v>-1.2</v>
       </c>
       <c r="G39" s="1">
         <f ca="1"/>
-        <v>-0.59999999999999987</v>
+        <v>-0.49999999999999978</v>
       </c>
       <c r="H39" s="1">
         <f ca="1"/>
-        <v>0.3</v>
+        <v>1.3</v>
       </c>
       <c r="I39" s="1">
         <f ca="1"/>
@@ -2943,7 +2946,7 @@
       </c>
       <c r="K39" s="1">
         <f ca="1"/>
-        <v>-1.5</v>
+        <v>-0.9</v>
       </c>
       <c r="L39" s="1">
         <f ca="1"/>
@@ -2951,39 +2954,39 @@
       </c>
       <c r="M39" s="1">
         <f ca="1"/>
-        <v>1.08</v>
+        <v>0</v>
       </c>
       <c r="N39" s="1">
         <f ca="1"/>
-        <v>-8.9999999999999969E-2</v>
+        <v>-5.9999999999999942E-2</v>
       </c>
       <c r="O39" s="1">
         <f ca="1"/>
-        <v>-1</v>
+        <v>0.1100000000000001</v>
       </c>
       <c r="P39" s="1">
         <f ca="1"/>
-        <v>0</v>
+        <v>-1.1399999999999999</v>
       </c>
       <c r="Q39" s="1">
         <f ca="1"/>
-        <v>-0.84999999999999987</v>
+        <v>-0.91999999999999993</v>
       </c>
       <c r="R39" s="1">
         <f ca="1"/>
-        <v>0.96</v>
+        <v>0.99</v>
       </c>
       <c r="S39" s="1">
         <f ca="1"/>
-        <v>1.21</v>
+        <v>1.19</v>
       </c>
       <c r="T39" s="1">
         <f ca="1"/>
-        <v>-1.23</v>
+        <v>-1.19</v>
       </c>
       <c r="U39" s="1">
         <f ca="1"/>
-        <v>-0.94999999999999984</v>
+        <v>-0.97999999999999987</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.35">
@@ -2992,7 +2995,7 @@
       </c>
       <c r="B41" s="1">
         <f t="shared" ref="B41:U41" ca="1" si="6">AVERAGE(B29:B39)</f>
-        <v>1</v>
+        <v>1.0000000000000002</v>
       </c>
       <c r="C41" s="1">
         <f t="shared" ca="1" si="6"/>
@@ -3012,11 +3015,11 @@
       </c>
       <c r="G41" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>-0.99999999999999989</v>
+        <v>-1</v>
       </c>
       <c r="H41" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>1.1000000000000001</v>
+        <v>1.0999999999999999</v>
       </c>
       <c r="I41" s="1">
         <f t="shared" ca="1" si="6"/>
@@ -3036,7 +3039,7 @@
       </c>
       <c r="M41" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>1.0000000000000002</v>
+        <v>0.99999999999999989</v>
       </c>
       <c r="N41" s="1">
         <f t="shared" ca="1" si="6"/>
@@ -3044,7 +3047,7 @@
       </c>
       <c r="O41" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>0</v>
+        <v>7.5697024406260668E-17</v>
       </c>
       <c r="P41" s="1">
         <f t="shared" ca="1" si="6"/>
@@ -3056,7 +3059,7 @@
       </c>
       <c r="R41" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>1.0999999999999999</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="S41" s="1">
         <f t="shared" ca="1" si="6"/>
@@ -3064,7 +3067,7 @@
       </c>
       <c r="T41" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>-1.1000000000000001</v>
+        <v>-1.0999999999999999</v>
       </c>
       <c r="U41" s="1">
         <f t="shared" ca="1" si="6"/>
@@ -3077,11 +3080,11 @@
       </c>
       <c r="B42" s="4">
         <f t="shared" ref="B42:U42" ca="1" si="7">_xlfn.STDEV.P(B29:B39)</f>
-        <v>0.63245553203367566</v>
+        <v>0.63245553203367544</v>
       </c>
       <c r="C42" s="4">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31622776601683844</v>
+        <v>0.31622776601683805</v>
       </c>
       <c r="D42" s="4">
         <f t="shared" ca="1" si="7"/>
@@ -3093,19 +3096,19 @@
       </c>
       <c r="F42" s="4">
         <f t="shared" ca="1" si="7"/>
-        <v>0.63245553203367588</v>
+        <v>0.6324555320336761</v>
       </c>
       <c r="G42" s="4">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31622776601683844</v>
+        <v>0.31622776601683783</v>
       </c>
       <c r="H42" s="4">
         <f t="shared" ca="1" si="7"/>
-        <v>0.63245553203367566</v>
+        <v>0.63245553203367588</v>
       </c>
       <c r="I42" s="4">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31622776601683783</v>
+        <v>0.31622776601683822</v>
       </c>
       <c r="J42" s="4">
         <f t="shared" ca="1" si="7"/>
@@ -3113,7 +3116,7 @@
       </c>
       <c r="K42" s="4">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31622776601683861</v>
+        <v>0.31622776601683822</v>
       </c>
       <c r="L42" s="1">
         <f t="shared" ca="1" si="7"/>
@@ -3121,11 +3124,11 @@
       </c>
       <c r="M42" s="1">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31780497164141358</v>
+        <v>0.31780497164141469</v>
       </c>
       <c r="N42" s="1">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31780497164141408</v>
+        <v>0.31780497164141402</v>
       </c>
       <c r="O42" s="1">
         <f t="shared" ca="1" si="7"/>
@@ -3141,19 +3144,19 @@
       </c>
       <c r="R42" s="1">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31780497164141486</v>
+        <v>0.31780497164141336</v>
       </c>
       <c r="S42" s="1">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31780497164141486</v>
+        <v>0.31780497164141414</v>
       </c>
       <c r="T42" s="1">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31780497164141375</v>
+        <v>0.31780497164141414</v>
       </c>
       <c r="U42" s="1">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31780497164141486</v>
+        <v>0.31780497164141414</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.35">
@@ -3162,35 +3165,35 @@
       </c>
       <c r="B43" s="1">
         <f t="shared" ref="B43:U43" ca="1" si="8">_xlfn.SKEW.P(B29:B39)</f>
-        <v>3.0278809762504267E-17</v>
+        <v>-1.0389416599759277E-15</v>
       </c>
       <c r="C43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>8.4780667335011958E-16</v>
+        <v>7.2669143430010251E-16</v>
       </c>
       <c r="D43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>-4.339962732625612E-16</v>
+        <v>-5.2483270255007403E-16</v>
       </c>
       <c r="E43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>4.0371746350005691E-16</v>
+        <v>4.8446095620006827E-16</v>
       </c>
       <c r="F43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>-4.1381040008755832E-16</v>
+        <v>-2.7124767078910076E-16</v>
       </c>
       <c r="G43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>-2.4223047810003414E-16</v>
+        <v>7.6706318065010816E-16</v>
       </c>
       <c r="H43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>-3.6334571715005125E-16</v>
+        <v>6.4531713306337224E-16</v>
       </c>
       <c r="I43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>1.1909665173251679E-15</v>
+        <v>1.1304088978001594E-15</v>
       </c>
       <c r="J43" s="1">
         <f t="shared" ca="1" si="8"/>
@@ -3198,27 +3201,27 @@
       </c>
       <c r="K43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>-5.6520444890007968E-16</v>
+        <v>-6.7118028306884468E-16</v>
       </c>
       <c r="L43" s="4">
         <f t="shared" ca="1" si="8"/>
-        <v>2.794540334892154</v>
+        <v>2.7945403348921536</v>
       </c>
       <c r="M43" s="4">
         <f t="shared" ca="1" si="8"/>
-        <v>-2.794540334892154</v>
+        <v>-2.7945403348921505</v>
       </c>
       <c r="N43" s="4">
         <f t="shared" ca="1" si="8"/>
-        <v>2.7945403348921518</v>
+        <v>2.7945403348921531</v>
       </c>
       <c r="O43" s="4">
         <f t="shared" ca="1" si="8"/>
-        <v>-2.7945403348921518</v>
+        <v>-2.7945403348921523</v>
       </c>
       <c r="P43" s="4">
         <f t="shared" ca="1" si="8"/>
-        <v>2.7945403348921536</v>
+        <v>2.794540334892154</v>
       </c>
       <c r="Q43" s="4">
         <f t="shared" ca="1" si="8"/>
@@ -3226,15 +3229,15 @@
       </c>
       <c r="R43" s="4">
         <f t="shared" ca="1" si="8"/>
-        <v>2.794540334892154</v>
+        <v>2.7945403348921518</v>
       </c>
       <c r="S43" s="4">
         <f t="shared" ca="1" si="8"/>
-        <v>-2.7945403348921505</v>
+        <v>-2.7945403348921518</v>
       </c>
       <c r="T43" s="4">
         <f t="shared" ca="1" si="8"/>
-        <v>2.794540334892154</v>
+        <v>2.7945403348921518</v>
       </c>
       <c r="U43" s="4">
         <f t="shared" ca="1" si="8"/>
@@ -3251,11 +3254,11 @@
       </c>
       <c r="C44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>-1.200000000000002</v>
+        <v>-1.2000000000000015</v>
       </c>
       <c r="D44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>-1.2000000000000011</v>
+        <v>-1.1999999999999997</v>
       </c>
       <c r="E44" s="1">
         <f t="shared" ca="1" si="9"/>
@@ -3271,11 +3274,11 @@
       </c>
       <c r="H44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>-1.200000000000002</v>
+        <v>-1.2000000000000002</v>
       </c>
       <c r="I44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>-1.2000000000000011</v>
+        <v>-1.2000000000000002</v>
       </c>
       <c r="J44" s="1">
         <f t="shared" ca="1" si="9"/>
@@ -3287,39 +3290,39 @@
       </c>
       <c r="L44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993706</v>
+        <v>10.711250530993702</v>
       </c>
       <c r="M44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993706</v>
+        <v>10.711250530993684</v>
       </c>
       <c r="N44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993684</v>
+        <v>10.711250530993706</v>
       </c>
       <c r="O44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993684</v>
+        <v>10.711250530993688</v>
       </c>
       <c r="P44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993702</v>
+        <v>10.711250530993706</v>
       </c>
       <c r="Q44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993706</v>
+        <v>10.711250530993702</v>
       </c>
       <c r="R44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993706</v>
+        <v>10.711250530993688</v>
       </c>
       <c r="S44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993684</v>
+        <v>10.711250530993695</v>
       </c>
       <c r="T44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993706</v>
+        <v>10.711250530993691</v>
       </c>
       <c r="U44" s="1">
         <f t="shared" ca="1" si="9"/>
@@ -3502,43 +3505,43 @@
       </c>
       <c r="B47" s="1">
         <f ca="1">CORREL(B29:B39,C29:C39)</f>
-        <v>0.12727272727272737</v>
+        <v>-0.21818181818181812</v>
       </c>
       <c r="D47" s="1">
         <f ca="1">CORREL(D29:D39,E29:E39)</f>
-        <v>-0.29090909090909095</v>
+        <v>-0.30909090909090897</v>
       </c>
       <c r="F47" s="1">
         <f ca="1">CORREL(F29:F39,G29:G39)</f>
-        <v>-0.33636363636363636</v>
+        <v>6.3636363636363588E-2</v>
       </c>
       <c r="H47" s="1">
         <f ca="1">CORREL(H29:H39,I29:I39)</f>
-        <v>0.2</v>
+        <v>6.3636363636363519E-2</v>
       </c>
       <c r="J47" s="1">
         <f ca="1">CORREL(J29:J39,K29:K39)</f>
-        <v>0.46363636363636357</v>
+        <v>-0.28181818181818186</v>
       </c>
       <c r="L47" s="1">
         <f ca="1">CORREL(L29:L39,M29:M39)</f>
-        <v>0.18712871287128705</v>
+        <v>0.10126012601260134</v>
       </c>
       <c r="N47" s="1">
         <f ca="1">CORREL(N29:N39,O29:O39)</f>
-        <v>9.9549954995499568E-2</v>
+        <v>0.10513051305130515</v>
       </c>
       <c r="P47" s="1">
         <f ca="1">CORREL(P29:P39,Q29:Q39)</f>
-        <v>0.12934293429342944</v>
+        <v>0.1245724572457247</v>
       </c>
       <c r="R47" s="1">
         <f ca="1">CORREL(R29:R39,S29:S39)</f>
-        <v>2.8352835283528287E-2</v>
+        <v>0.12763276327632767</v>
       </c>
       <c r="T47" s="1">
         <f ca="1">CORREL(T29:T39,U29:U39)</f>
-        <v>0.1224122412241225</v>
+        <v>2.1062106210620948E-2</v>
       </c>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.35">
@@ -3547,27 +3550,27 @@
       </c>
       <c r="B48">
         <f t="array" aca="1" ref="B48" ca="1">SUMPRODUCT((B29:B39&gt;C29:C39)*1)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C48">
         <f t="array" aca="1" ref="C48" ca="1">SUMPRODUCT((B29:B39&lt;C29:C39)*1)</f>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D48">
         <f t="array" aca="1" ref="D48" ca="1">SUMPRODUCT((D29:D39&gt;E29:E39)*1)</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E48">
         <f t="array" aca="1" ref="E48" ca="1">SUMPRODUCT((D29:D39&lt;E29:E39)*1)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F48">
         <f t="array" aca="1" ref="F48" ca="1">SUMPRODUCT((F29:F39&gt;G29:G39)*1)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G48">
         <f t="array" aca="1" ref="G48" ca="1">SUMPRODUCT((F29:F39&lt;G29:G39)*1)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H48">
         <f t="array" aca="1" ref="H48" ca="1">SUMPRODUCT((H29:H39&gt;I29:I39)*1)</f>
@@ -3575,15 +3578,15 @@
       </c>
       <c r="I48">
         <f t="array" aca="1" ref="I48" ca="1">SUMPRODUCT((H29:H39&lt;I29:I39)*1)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J48">
         <f t="array" aca="1" ref="J48" ca="1">SUMPRODUCT((J29:J39&gt;K29:K39)*1)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K48">
         <f t="array" aca="1" ref="K48" ca="1">SUMPRODUCT((J29:J39&lt;K29:K39)*1)</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L48">
         <f t="array" aca="1" ref="L48" ca="1">SUMPRODUCT((L29:L39&gt;M29:M39)*1)</f>
@@ -3632,15 +3635,15 @@
       </c>
       <c r="B49" s="6" t="str">
         <f ca="1">IF(B48&gt;C48,"A",IF(C48&gt;B48,"B","Equal"))</f>
-        <v>B</v>
+        <v>A</v>
       </c>
       <c r="D49" s="6" t="str">
         <f ca="1">IF(D48&gt;E48,"A",IF(E48&gt;D48,"B","Equal"))</f>
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="F49" s="6" t="str">
         <f ca="1">IF(F48&gt;G48,"A",IF(G48&gt;F48,"B","Equal"))</f>
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="H49" s="6" t="str">
         <f ca="1">IF(H48&gt;I48,"A",IF(I48&gt;H48,"B","Equal"))</f>
@@ -3648,7 +3651,7 @@
       </c>
       <c r="J49" s="6" t="str">
         <f ca="1">IF(J48&gt;K48,"A",IF(K48&gt;J48,"B","Equal"))</f>
-        <v>B</v>
+        <v>A</v>
       </c>
       <c r="L49" s="6" t="str">
         <f ca="1">IF(L48&gt;M48,"A",IF(M48&gt;L48,"B","Equal"))</f>
@@ -3681,7 +3684,7 @@
       </c>
       <c r="D50">
         <f ca="1">MAX(D48:E48)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F50">
         <f ca="1">MAX(F48:G48)</f>
@@ -6743,8 +6746,11 @@
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A104" s="8" t="s">
-        <v>24</v>
-      </c>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="105" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A105" s="8"/>
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.35">
       <c r="B106" s="8" t="s">
@@ -6780,7 +6786,7 @@
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A107" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B107" s="10">
         <v>0.8</v>
@@ -6815,7 +6821,7 @@
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A108" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B108" s="10">
         <v>0.6</v>
@@ -6850,7 +6856,7 @@
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A109" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B109" s="10">
         <v>1.4</v>
@@ -6881,6 +6887,41 @@
       </c>
       <c r="T109" s="10">
         <v>1.4</v>
+      </c>
+    </row>
+    <row r="110" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A110" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B110" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="D110" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="F110" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="H110" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="J110" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="L110" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="N110" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="P110" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="R110" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="T110" s="10">
+        <v>1.2</v>
       </c>
     </row>
   </sheetData>
@@ -6890,7 +6931,6 @@
     <mergeCell ref="D54:E54"/>
     <mergeCell ref="P54:Q54"/>
     <mergeCell ref="T54:U54"/>
-    <mergeCell ref="D2:E2"/>
     <mergeCell ref="F80:G80"/>
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="P2:Q2"/>
@@ -6905,14 +6945,15 @@
     <mergeCell ref="L54:M54"/>
     <mergeCell ref="R54:S54"/>
     <mergeCell ref="N28:O28"/>
+    <mergeCell ref="F28:G28"/>
     <mergeCell ref="R28:S28"/>
     <mergeCell ref="J28:K28"/>
     <mergeCell ref="D80:E80"/>
     <mergeCell ref="L28:M28"/>
     <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="D28:E28"/>
-    <mergeCell ref="F28:G28"/>
     <mergeCell ref="P28:Q28"/>
     <mergeCell ref="H28:I28"/>
     <mergeCell ref="H80:I80"/>

</xml_diff>

<commit_message>
set equl L/H values
</commit_message>
<xml_diff>
--- a/Distributions.xlsx
+++ b/Distributions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aaltofi-my.sharepoint.com/personal/samuel_salin_aalto_fi/Documents/Desktop/Risk Elicitation/RE/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/svsalin/Desktop/Risk Elicitation/RE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_BA4D2FB74CA8045DC74C1AC6005315D59D888FE4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E53CF80-D76A-45FC-B8D4-F6B92E7F8969}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4561273A-B9FF-774F-B9CF-5D9C1A4A8399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5160" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21160" yWindow="-28800" windowWidth="68800" windowHeight="28800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All" sheetId="1" r:id="rId1"/>
@@ -544,12 +544,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:AB110"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="198.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="198.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
       <c r="B2" s="11" t="s">
         <v>0</v>
@@ -592,7 +592,7 @@
       </c>
       <c r="U2" s="12"/>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B3" s="1">
         <v>0</v>
       </c>
@@ -654,7 +654,7 @@
         <v>-1.05</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B4" s="1">
         <v>0.2</v>
       </c>
@@ -716,7 +716,7 @@
         <v>-1.04</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B5" s="1">
         <v>0.4</v>
       </c>
@@ -778,7 +778,7 @@
         <v>-1.03</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B6" s="1">
         <v>0.60000000000000009</v>
       </c>
@@ -840,7 +840,7 @@
         <v>-1.02</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B7" s="1">
         <v>0.8</v>
       </c>
@@ -902,7 +902,7 @@
         <v>-1.01</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B8" s="1">
         <v>1</v>
       </c>
@@ -964,7 +964,7 @@
         <v>-0.98999999999999988</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B9" s="1">
         <v>1.2</v>
       </c>
@@ -1026,7 +1026,7 @@
         <v>-0.97999999999999987</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B10" s="1">
         <v>1.4</v>
       </c>
@@ -1088,7 +1088,7 @@
         <v>-0.96999999999999986</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B11" s="1">
         <v>1.6</v>
       </c>
@@ -1150,7 +1150,7 @@
         <v>-0.95999999999999985</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B12" s="1">
         <v>1.8</v>
       </c>
@@ -1212,7 +1212,7 @@
         <v>-0.94999999999999984</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B13" s="1">
         <v>2</v>
       </c>
@@ -1274,7 +1274,7 @@
         <v>-2.1</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -1359,7 +1359,7 @@
         <v>-1.0999999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>11</v>
       </c>
@@ -1444,7 +1444,7 @@
         <v>0.31780497164141486</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>-2.7945403348921518</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -1614,7 +1614,7 @@
         <v>10.711250530993691</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>14</v>
       </c>
@@ -1699,7 +1699,7 @@
         <v>-2.1</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>15</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>-0.94999999999999984</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -1829,7 +1829,7 @@
         <v>-0.98019801980197996</v>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>17</v>
       </c>
@@ -1914,7 +1914,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
         <v>18</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>B</v>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>19</v>
       </c>
@@ -2004,12 +2004,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>21</v>
       </c>
@@ -2054,17 +2054,17 @@
       </c>
       <c r="U28" s="12"/>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>1</v>
       </c>
       <c r="B29" s="1">
         <f t="array" aca="1" ref="B29:B39" ca="1">_xlfn.SORTBY(B3:B13,_xlfn.RANDARRAY(ROWS(B3:B13)))</f>
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="C29" s="1">
         <f t="array" aca="1" ref="C29:C39" ca="1">_xlfn.SORTBY(C3:C13,_xlfn.RANDARRAY(ROWS(C3:C13)))</f>
-        <v>0.79999999999999993</v>
+        <v>1.4</v>
       </c>
       <c r="D29" s="1">
         <f t="array" aca="1" ref="D29:D39" ca="1">_xlfn.SORTBY(D3:D13,_xlfn.RANDARRAY(ROWS(D3:D13)))</f>
@@ -2072,51 +2072,51 @@
       </c>
       <c r="E29" s="1">
         <f t="array" aca="1" ref="E29:E39" ca="1">_xlfn.SORTBY(E3:E13,_xlfn.RANDARRAY(ROWS(E3:E13)))</f>
-        <v>9.9999999999999867E-2</v>
+        <v>-0.4</v>
       </c>
       <c r="F29" s="1">
         <f t="array" aca="1" ref="F29:F39" ca="1">_xlfn.SORTBY(F3:F13,_xlfn.RANDARRAY(ROWS(F3:F13)))</f>
-        <v>-2</v>
+        <v>-0.60000000000000009</v>
       </c>
       <c r="G29" s="1">
         <f t="array" aca="1" ref="G29:G39" ca="1">_xlfn.SORTBY(G3:G13,_xlfn.RANDARRAY(ROWS(G3:G13)))</f>
-        <v>-0.59999999999999987</v>
+        <v>-0.90000000000000013</v>
       </c>
       <c r="H29" s="1">
         <f t="array" aca="1" ref="H29:H39" ca="1">_xlfn.SORTBY(H3:H13,_xlfn.RANDARRAY(ROWS(H3:H13)))</f>
-        <v>1.1000000000000001</v>
+        <v>1.3</v>
       </c>
       <c r="I29" s="1">
         <f t="array" aca="1" ref="I29:I39" ca="1">_xlfn.SORTBY(I3:I13,_xlfn.RANDARRAY(ROWS(I3:I13)))</f>
-        <v>0.79999999999999993</v>
+        <v>0.7</v>
       </c>
       <c r="J29" s="1">
         <f t="array" aca="1" ref="J29:J39" ca="1">_xlfn.SORTBY(J3:J13,_xlfn.RANDARRAY(ROWS(J3:J13)))</f>
-        <v>-1.9</v>
+        <v>-0.9</v>
       </c>
       <c r="K29" s="1">
         <f t="array" aca="1" ref="K29:K39" ca="1">_xlfn.SORTBY(K3:K13,_xlfn.RANDARRAY(ROWS(K3:K13)))</f>
-        <v>-0.59999999999999976</v>
+        <v>-1.5</v>
       </c>
       <c r="L29" s="1">
         <f t="array" aca="1" ref="L29:L39" ca="1">_xlfn.SORTBY(L3:L13,_xlfn.RANDARRAY(ROWS(L3:L13)))</f>
-        <v>0.89</v>
+        <v>0.95000000000000007</v>
       </c>
       <c r="M29" s="1">
         <f t="array" aca="1" ref="M29:M39" ca="1">_xlfn.SORTBY(M3:M13,_xlfn.RANDARRAY(ROWS(M3:M13)))</f>
-        <v>1.07</v>
+        <v>0</v>
       </c>
       <c r="N29" s="1">
         <f t="array" aca="1" ref="N29:N39" ca="1">_xlfn.SORTBY(N3:N13,_xlfn.RANDARRAY(ROWS(N3:N13)))</f>
-        <v>1</v>
+        <v>-5.9999999999999942E-2</v>
       </c>
       <c r="O29" s="1">
         <f t="array" aca="1" ref="O29:O39" ca="1">_xlfn.SORTBY(O3:O13,_xlfn.RANDARRAY(ROWS(O3:O13)))</f>
-        <v>0.12000000000000011</v>
+        <v>9.000000000000008E-2</v>
       </c>
       <c r="P29" s="1">
         <f t="array" aca="1" ref="P29:P39" ca="1">_xlfn.SORTBY(P3:P13,_xlfn.RANDARRAY(ROWS(P3:P13)))</f>
-        <v>-1.05</v>
+        <v>-1.07</v>
       </c>
       <c r="Q29" s="1">
         <f t="array" aca="1" ref="Q29:Q39" ca="1">_xlfn.SORTBY(Q3:Q13,_xlfn.RANDARRAY(ROWS(Q3:Q13)))</f>
@@ -2124,22 +2124,22 @@
       </c>
       <c r="R29" s="1">
         <f t="array" aca="1" ref="R29:R39" ca="1">_xlfn.SORTBY(R3:R13,_xlfn.RANDARRAY(ROWS(R3:R13)))</f>
-        <v>0.95</v>
+        <v>0.97</v>
       </c>
       <c r="S29" s="1">
         <f t="array" aca="1" ref="S29:S39" ca="1">_xlfn.SORTBY(S3:S13,_xlfn.RANDARRAY(ROWS(S3:S13)))</f>
-        <v>1.23</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="T29" s="1">
         <f t="array" aca="1" ref="T29:T39" ca="1">_xlfn.SORTBY(T3:T13,_xlfn.RANDARRAY(ROWS(T3:T13)))</f>
-        <v>-1.1599999999999999</v>
+        <v>-1.18</v>
       </c>
       <c r="U29" s="1">
         <f t="array" aca="1" ref="U29:U39" ca="1">_xlfn.SORTBY(U3:U13,_xlfn.RANDARRAY(ROWS(U3:U13)))</f>
-        <v>-2.1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.35">
+        <v>-0.95999999999999985</v>
+      </c>
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>2</v>
       </c>
@@ -2149,59 +2149,59 @@
       </c>
       <c r="C30" s="1">
         <f ca="1"/>
+        <v>1.2</v>
+      </c>
+      <c r="D30" s="1">
+        <f ca="1"/>
+        <v>-0.39999999999999991</v>
+      </c>
+      <c r="E30" s="1">
+        <f ca="1"/>
+        <v>-0.1000000000000001</v>
+      </c>
+      <c r="F30" s="1">
+        <f ca="1"/>
+        <v>-0.8</v>
+      </c>
+      <c r="G30" s="1">
+        <f ca="1"/>
+        <v>-0.59999999999999987</v>
+      </c>
+      <c r="H30" s="1">
+        <f ca="1"/>
+        <v>1.9</v>
+      </c>
+      <c r="I30" s="1">
+        <f ca="1"/>
         <v>1.1000000000000001</v>
       </c>
-      <c r="D30" s="1">
-        <f ca="1"/>
-        <v>-0.2</v>
-      </c>
-      <c r="E30" s="1">
-        <f ca="1"/>
-        <v>0.40000000000000008</v>
-      </c>
-      <c r="F30" s="1">
-        <f ca="1"/>
-        <v>-1</v>
-      </c>
-      <c r="G30" s="1">
-        <f ca="1"/>
-        <v>-0.8</v>
-      </c>
-      <c r="H30" s="1">
-        <f ca="1"/>
-        <v>0.5</v>
-      </c>
-      <c r="I30" s="1">
-        <f ca="1"/>
-        <v>1.1000000000000001</v>
-      </c>
       <c r="J30" s="1">
         <f ca="1"/>
-        <v>-0.70000000000000007</v>
+        <v>-0.30000000000000021</v>
       </c>
       <c r="K30" s="1">
         <f ca="1"/>
-        <v>-1.5</v>
+        <v>-0.79999999999999993</v>
       </c>
       <c r="L30" s="1">
         <f ca="1"/>
-        <v>0.85</v>
+        <v>0.93</v>
       </c>
       <c r="M30" s="1">
         <f ca="1"/>
-        <v>1.08</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="N30" s="1">
         <f ca="1"/>
-        <v>-0.12</v>
+        <v>-7.999999999999996E-2</v>
       </c>
       <c r="O30" s="1">
         <f ca="1"/>
-        <v>5.0000000000000037E-2</v>
+        <v>6.0000000000000053E-2</v>
       </c>
       <c r="P30" s="1">
         <f ca="1"/>
-        <v>0</v>
+        <v>-1.05</v>
       </c>
       <c r="Q30" s="1">
         <f ca="1"/>
@@ -2209,28 +2209,28 @@
       </c>
       <c r="R30" s="1">
         <f ca="1"/>
-        <v>1.01</v>
+        <v>0.96</v>
       </c>
       <c r="S30" s="1">
         <f ca="1"/>
-        <v>0.1</v>
+        <v>1.17</v>
       </c>
       <c r="T30" s="1">
         <f ca="1"/>
-        <v>-1.25</v>
+        <v>-1.22</v>
       </c>
       <c r="U30" s="1">
         <f ca="1"/>
         <v>-0.96999999999999986</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>3</v>
       </c>
       <c r="B31" s="1">
         <f ca="1"/>
-        <v>0.60000000000000009</v>
+        <v>0.4</v>
       </c>
       <c r="C31" s="1">
         <f ca="1"/>
@@ -2238,43 +2238,43 @@
       </c>
       <c r="D31" s="1">
         <f ca="1"/>
+        <v>0</v>
+      </c>
+      <c r="E31" s="1">
+        <f ca="1"/>
+        <v>0.50000000000000022</v>
+      </c>
+      <c r="F31" s="1">
+        <f ca="1"/>
+        <v>-0.40000000000000008</v>
+      </c>
+      <c r="G31" s="1">
+        <f ca="1"/>
+        <v>-0.8</v>
+      </c>
+      <c r="H31" s="1">
+        <f ca="1"/>
+        <v>0.70000000000000007</v>
+      </c>
+      <c r="I31" s="1">
+        <f ca="1"/>
+        <v>0.99999999999999989</v>
+      </c>
+      <c r="J31" s="1">
+        <f ca="1"/>
+        <v>-1.3</v>
+      </c>
+      <c r="K31" s="1">
+        <f ca="1"/>
         <v>-1</v>
       </c>
-      <c r="E31" s="1">
-        <f ca="1"/>
-        <v>-0.20000000000000009</v>
-      </c>
-      <c r="F31" s="1">
-        <f ca="1"/>
-        <v>-0.60000000000000009</v>
-      </c>
-      <c r="G31" s="1">
-        <f ca="1"/>
-        <v>-1.2</v>
-      </c>
-      <c r="H31" s="1">
-        <f ca="1"/>
-        <v>1.5</v>
-      </c>
-      <c r="I31" s="1">
-        <f ca="1"/>
-        <v>1.2</v>
-      </c>
-      <c r="J31" s="1">
-        <f ca="1"/>
-        <v>-0.50000000000000011</v>
-      </c>
-      <c r="K31" s="1">
-        <f ca="1"/>
-        <v>-0.79999999999999993</v>
-      </c>
       <c r="L31" s="1">
         <f ca="1"/>
         <v>0.88</v>
       </c>
       <c r="M31" s="1">
         <f ca="1"/>
-        <v>1.1399999999999999</v>
+        <v>1.06</v>
       </c>
       <c r="N31" s="1">
         <f ca="1"/>
@@ -2290,36 +2290,36 @@
       </c>
       <c r="Q31" s="1">
         <f ca="1"/>
-        <v>-0.87999999999999989</v>
+        <v>-0.85999999999999988</v>
       </c>
       <c r="R31" s="1">
         <f ca="1"/>
-        <v>2.1</v>
+        <v>1.03</v>
       </c>
       <c r="S31" s="1">
         <f ca="1"/>
-        <v>1.24</v>
+        <v>1.21</v>
       </c>
       <c r="T31" s="1">
         <f ca="1"/>
-        <v>-1.22</v>
+        <v>-1.21</v>
       </c>
       <c r="U31" s="1">
         <f ca="1"/>
-        <v>-0.95999999999999985</v>
-      </c>
-    </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.35">
+        <v>-0.98999999999999988</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>4</v>
       </c>
       <c r="B32" s="1">
         <f ca="1"/>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="C32" s="1">
         <f ca="1"/>
-        <v>0.99999999999999989</v>
+        <v>0.6</v>
       </c>
       <c r="D32" s="1">
         <f ca="1"/>
@@ -2327,159 +2327,159 @@
       </c>
       <c r="E32" s="1">
         <f ca="1"/>
+        <v>9.9999999999999867E-2</v>
+      </c>
+      <c r="F32" s="1">
+        <f ca="1"/>
+        <v>-1.8</v>
+      </c>
+      <c r="G32" s="1">
+        <f ca="1"/>
+        <v>-1</v>
+      </c>
+      <c r="H32" s="1">
+        <f ca="1"/>
+        <v>0.5</v>
+      </c>
+      <c r="I32" s="1">
+        <f ca="1"/>
+        <v>1.2</v>
+      </c>
+      <c r="J32" s="1">
+        <f ca="1"/>
+        <v>-1.1000000000000001</v>
+      </c>
+      <c r="K32" s="1">
+        <f ca="1"/>
+        <v>-0.59999999999999976</v>
+      </c>
+      <c r="L32" s="1">
+        <f ca="1"/>
+        <v>0.89</v>
+      </c>
+      <c r="M32" s="1">
+        <f ca="1"/>
+        <v>1.07</v>
+      </c>
+      <c r="N32" s="1">
+        <f ca="1"/>
+        <v>-4.9999999999999933E-2</v>
+      </c>
+      <c r="O32" s="1">
+        <f ca="1"/>
+        <v>0.15000000000000011</v>
+      </c>
+      <c r="P32" s="1">
+        <f ca="1"/>
         <v>0</v>
       </c>
-      <c r="F32" s="1">
-        <f ca="1"/>
-        <v>-1.4</v>
-      </c>
-      <c r="G32" s="1">
-        <f ca="1"/>
-        <v>-0.90000000000000013</v>
-      </c>
-      <c r="H32" s="1">
-        <f ca="1"/>
-        <v>0.3</v>
-      </c>
-      <c r="I32" s="1">
-        <f ca="1"/>
-        <v>0.99999999999999989</v>
-      </c>
-      <c r="J32" s="1">
-        <f ca="1"/>
-        <v>-1.3</v>
-      </c>
-      <c r="K32" s="1">
-        <f ca="1"/>
-        <v>-1.3</v>
-      </c>
-      <c r="L32" s="1">
-        <f ca="1"/>
-        <v>0.92</v>
-      </c>
-      <c r="M32" s="1">
-        <f ca="1"/>
-        <v>1.05</v>
-      </c>
-      <c r="N32" s="1">
-        <f ca="1"/>
-        <v>-4.9999999999999933E-2</v>
-      </c>
-      <c r="O32" s="1">
-        <f ca="1"/>
-        <v>7.0000000000000062E-2</v>
-      </c>
-      <c r="P32" s="1">
-        <f ca="1"/>
-        <v>-1.06</v>
-      </c>
       <c r="Q32" s="1">
         <f ca="1"/>
-        <v>-0.95</v>
+        <v>-0.87999999999999989</v>
       </c>
       <c r="R32" s="1">
         <f ca="1"/>
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="S32" s="1">
         <f ca="1"/>
-        <v>1.21</v>
+        <v>1.24</v>
       </c>
       <c r="T32" s="1">
         <f ca="1"/>
-        <v>-1.24</v>
+        <v>-1.23</v>
       </c>
       <c r="U32" s="1">
         <f ca="1"/>
         <v>-1.03</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>5</v>
       </c>
       <c r="B33" s="1">
         <f ca="1"/>
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="C33" s="1">
         <f ca="1"/>
+        <v>0.99999999999999989</v>
+      </c>
+      <c r="D33" s="1">
+        <f ca="1"/>
+        <v>-0.8</v>
+      </c>
+      <c r="E33" s="1">
+        <f ca="1"/>
+        <v>-0.3</v>
+      </c>
+      <c r="F33" s="1">
+        <f ca="1"/>
+        <v>-0.20000000000000021</v>
+      </c>
+      <c r="G33" s="1">
+        <f ca="1"/>
+        <v>-1.5</v>
+      </c>
+      <c r="H33" s="1">
+        <f ca="1"/>
+        <v>0.3</v>
+      </c>
+      <c r="I33" s="1">
+        <f ca="1"/>
         <v>0.89999999999999991</v>
       </c>
-      <c r="D33" s="1">
-        <f ca="1"/>
-        <v>-0.8</v>
-      </c>
-      <c r="E33" s="1">
-        <f ca="1"/>
-        <v>-0.1000000000000001</v>
-      </c>
-      <c r="F33" s="1">
-        <f ca="1"/>
-        <v>-0.20000000000000021</v>
-      </c>
-      <c r="G33" s="1">
-        <f ca="1"/>
-        <v>-0.7</v>
-      </c>
-      <c r="H33" s="1">
-        <f ca="1"/>
-        <v>1.9</v>
-      </c>
-      <c r="I33" s="1">
-        <f ca="1"/>
-        <v>1.4</v>
-      </c>
       <c r="J33" s="1">
         <f ca="1"/>
-        <v>-2.1</v>
+        <v>-0.50000000000000011</v>
       </c>
       <c r="K33" s="1">
         <f ca="1"/>
-        <v>-1</v>
+        <v>-1.6</v>
       </c>
       <c r="L33" s="1">
         <f ca="1"/>
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
       <c r="M33" s="1">
         <f ca="1"/>
-        <v>1.1299999999999999</v>
+        <v>1.08</v>
       </c>
       <c r="N33" s="1">
         <f ca="1"/>
-        <v>-0.11</v>
+        <v>1</v>
       </c>
       <c r="O33" s="1">
         <f ca="1"/>
-        <v>8.0000000000000071E-2</v>
+        <v>5.0000000000000037E-2</v>
       </c>
       <c r="P33" s="1">
         <f ca="1"/>
-        <v>-1.1299999999999999</v>
+        <v>-1.0900000000000001</v>
       </c>
       <c r="Q33" s="1">
         <f ca="1"/>
-        <v>-0.8899999999999999</v>
+        <v>-0.90999999999999992</v>
       </c>
       <c r="R33" s="1">
         <f ca="1"/>
-        <v>1.03</v>
+        <v>1.02</v>
       </c>
       <c r="S33" s="1">
         <f ca="1"/>
-        <v>1.25</v>
+        <v>0.1</v>
       </c>
       <c r="T33" s="1">
         <f ca="1"/>
-        <v>-1.23</v>
+        <v>-1.25</v>
       </c>
       <c r="U33" s="1">
         <f ca="1"/>
-        <v>-1.05</v>
-      </c>
-    </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.35">
+        <v>-1.01</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>6</v>
       </c>
@@ -2493,15 +2493,15 @@
       </c>
       <c r="D34" s="1">
         <f ca="1"/>
-        <v>0.2</v>
+        <v>0.59999999999999987</v>
       </c>
       <c r="E34" s="1">
         <f ca="1"/>
-        <v>0.3</v>
+        <v>-0.5</v>
       </c>
       <c r="F34" s="1">
         <f ca="1"/>
-        <v>-1.6</v>
+        <v>-2</v>
       </c>
       <c r="G34" s="1">
         <f ca="1"/>
@@ -2509,11 +2509,11 @@
       </c>
       <c r="H34" s="1">
         <f ca="1"/>
-        <v>0.70000000000000007</v>
+        <v>0.1</v>
       </c>
       <c r="I34" s="1">
         <f ca="1"/>
-        <v>0.6</v>
+        <v>0.79999999999999993</v>
       </c>
       <c r="J34" s="1">
         <f ca="1"/>
@@ -2521,15 +2521,15 @@
       </c>
       <c r="K34" s="1">
         <f ca="1"/>
-        <v>-1.4</v>
+        <v>-0.9</v>
       </c>
       <c r="L34" s="1">
         <f ca="1"/>
-        <v>0.95000000000000007</v>
+        <v>0.92</v>
       </c>
       <c r="M34" s="1">
         <f ca="1"/>
-        <v>1.1499999999999999</v>
+        <v>1.0900000000000001</v>
       </c>
       <c r="N34" s="1">
         <f ca="1"/>
@@ -2537,80 +2537,80 @@
       </c>
       <c r="O34" s="1">
         <f ca="1"/>
-        <v>9.000000000000008E-2</v>
+        <v>7.0000000000000062E-2</v>
       </c>
       <c r="P34" s="1">
         <f ca="1"/>
-        <v>-1.1200000000000001</v>
+        <v>-1.1100000000000001</v>
       </c>
       <c r="Q34" s="1">
         <f ca="1"/>
-        <v>-0.85999999999999988</v>
+        <v>-2</v>
       </c>
       <c r="R34" s="1">
         <f ca="1"/>
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="S34" s="1">
         <f ca="1"/>
-        <v>1.18</v>
+        <v>1.23</v>
       </c>
       <c r="T34" s="1">
         <f ca="1"/>
-        <v>-1.21</v>
+        <v>-1.17</v>
       </c>
       <c r="U34" s="1">
         <f ca="1"/>
-        <v>-1.01</v>
-      </c>
-    </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.35">
+        <v>-0.97999999999999987</v>
+      </c>
+    </row>
+    <row r="35" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>7</v>
       </c>
       <c r="B35" s="1">
         <f ca="1"/>
+        <v>1</v>
+      </c>
+      <c r="C35" s="1">
+        <f ca="1"/>
+        <v>0.5</v>
+      </c>
+      <c r="D35" s="1">
+        <f ca="1"/>
+        <v>-1</v>
+      </c>
+      <c r="E35" s="1">
+        <f ca="1"/>
         <v>0.2</v>
       </c>
-      <c r="C35" s="1">
-        <f ca="1"/>
-        <v>1.2</v>
-      </c>
-      <c r="D35" s="1">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="E35" s="1">
-        <f ca="1"/>
-        <v>0.2</v>
-      </c>
       <c r="F35" s="1">
         <f ca="1"/>
-        <v>-0.8</v>
+        <v>-1</v>
       </c>
       <c r="G35" s="1">
         <f ca="1"/>
-        <v>-1.3</v>
+        <v>-1.1000000000000001</v>
       </c>
       <c r="H35" s="1">
         <f ca="1"/>
-        <v>1.7</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="I35" s="1">
         <f ca="1"/>
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
       <c r="J35" s="1">
         <f ca="1"/>
-        <v>-0.30000000000000021</v>
+        <v>-1.7</v>
       </c>
       <c r="K35" s="1">
         <f ca="1"/>
-        <v>-0.69999999999999984</v>
+        <v>-1.1000000000000001</v>
       </c>
       <c r="L35" s="1">
         <f ca="1"/>
-        <v>0.94000000000000006</v>
+        <v>0.86</v>
       </c>
       <c r="M35" s="1">
         <f ca="1"/>
@@ -2618,38 +2618,38 @@
       </c>
       <c r="N35" s="1">
         <f ca="1"/>
-        <v>-6.9999999999999951E-2</v>
+        <v>-0.12</v>
       </c>
       <c r="O35" s="1">
         <f ca="1"/>
-        <v>6.0000000000000053E-2</v>
+        <v>8.0000000000000071E-2</v>
       </c>
       <c r="P35" s="1">
         <f ca="1"/>
-        <v>-1.07</v>
+        <v>-1.1299999999999999</v>
       </c>
       <c r="Q35" s="1">
         <f ca="1"/>
-        <v>-0.86999999999999988</v>
+        <v>-0.8899999999999999</v>
       </c>
       <c r="R35" s="1">
         <f ca="1"/>
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
       <c r="S35" s="1">
         <f ca="1"/>
-        <v>1.17</v>
+        <v>1.18</v>
       </c>
       <c r="T35" s="1">
         <f ca="1"/>
-        <v>-1.17</v>
+        <v>-1.1499999999999999</v>
       </c>
       <c r="U35" s="1">
         <f ca="1"/>
-        <v>-0.94999999999999984</v>
-      </c>
-    </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.35">
+        <v>-2.1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>8</v>
       </c>
@@ -2659,92 +2659,92 @@
       </c>
       <c r="C36" s="1">
         <f ca="1"/>
-        <v>1.4</v>
+        <v>0.79999999999999993</v>
       </c>
       <c r="D36" s="1">
         <f ca="1"/>
-        <v>-0.39999999999999991</v>
+        <v>0.99999999999999978</v>
       </c>
       <c r="E36" s="1">
         <f ca="1"/>
-        <v>0.50000000000000022</v>
+        <v>-0.20000000000000009</v>
       </c>
       <c r="F36" s="1">
         <f ca="1"/>
-        <v>-0.40000000000000008</v>
+        <v>0</v>
       </c>
       <c r="G36" s="1">
         <f ca="1"/>
-        <v>-1.1000000000000001</v>
+        <v>-0.7</v>
       </c>
       <c r="H36" s="1">
         <f ca="1"/>
-        <v>0.9</v>
+        <v>1.7</v>
       </c>
       <c r="I36" s="1">
         <f ca="1"/>
-        <v>0.89999999999999991</v>
+        <v>1.6</v>
       </c>
       <c r="J36" s="1">
         <f ca="1"/>
-        <v>-0.9</v>
+        <v>-2.1</v>
       </c>
       <c r="K36" s="1">
         <f ca="1"/>
-        <v>-1.1000000000000001</v>
+        <v>-1.2</v>
       </c>
       <c r="L36" s="1">
         <f ca="1"/>
-        <v>0.87</v>
+        <v>0.94000000000000006</v>
       </c>
       <c r="M36" s="1">
         <f ca="1"/>
-        <v>1.06</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="N36" s="1">
         <f ca="1"/>
-        <v>-8.9999999999999969E-2</v>
+        <v>-0.11</v>
       </c>
       <c r="O36" s="1">
         <f ca="1"/>
-        <v>-1</v>
+        <v>0.12000000000000011</v>
       </c>
       <c r="P36" s="1">
         <f ca="1"/>
-        <v>-1.1100000000000001</v>
+        <v>-1.1200000000000001</v>
       </c>
       <c r="Q36" s="1">
         <f ca="1"/>
-        <v>-0.90999999999999992</v>
+        <v>-0.91999999999999993</v>
       </c>
       <c r="R36" s="1">
         <f ca="1"/>
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
       <c r="S36" s="1">
         <f ca="1"/>
-        <v>1.1499999999999999</v>
+        <v>1.25</v>
       </c>
       <c r="T36" s="1">
         <f ca="1"/>
-        <v>-0.1</v>
+        <v>-1.19</v>
       </c>
       <c r="U36" s="1">
         <f ca="1"/>
-        <v>-1.04</v>
-      </c>
-    </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.35">
+        <v>-1.05</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>9</v>
       </c>
       <c r="B37" s="1">
         <f ca="1"/>
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="C37" s="1">
         <f ca="1"/>
-        <v>0.5</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="D37" s="1">
         <f ca="1"/>
@@ -2752,128 +2752,128 @@
       </c>
       <c r="E37" s="1">
         <f ca="1"/>
-        <v>-0.3</v>
+        <v>0</v>
       </c>
       <c r="F37" s="1">
         <f ca="1"/>
-        <v>0</v>
+        <v>-1.2</v>
       </c>
       <c r="G37" s="1">
         <f ca="1"/>
+        <v>-0.49999999999999978</v>
+      </c>
+      <c r="H37" s="1">
+        <f ca="1"/>
+        <v>1.5</v>
+      </c>
+      <c r="I37" s="1">
+        <f ca="1"/>
+        <v>1.5</v>
+      </c>
+      <c r="J37" s="1">
+        <f ca="1"/>
+        <v>-0.1</v>
+      </c>
+      <c r="K37" s="1">
+        <f ca="1"/>
+        <v>-1.3</v>
+      </c>
+      <c r="L37" s="1">
+        <f ca="1"/>
+        <v>0.87</v>
+      </c>
+      <c r="M37" s="1">
+        <f ca="1"/>
+        <v>1.05</v>
+      </c>
+      <c r="N37" s="1">
+        <f ca="1"/>
+        <v>-0.14000000000000001</v>
+      </c>
+      <c r="O37" s="1">
+        <f ca="1"/>
         <v>-1</v>
       </c>
-      <c r="H37" s="1">
-        <f ca="1"/>
-        <v>0.1</v>
-      </c>
-      <c r="I37" s="1">
-        <f ca="1"/>
-        <v>1.5</v>
-      </c>
-      <c r="J37" s="1">
+      <c r="P37" s="1">
+        <f ca="1"/>
+        <v>-1.08</v>
+      </c>
+      <c r="Q37" s="1">
+        <f ca="1"/>
+        <v>-0.95</v>
+      </c>
+      <c r="R37" s="1">
+        <f ca="1"/>
+        <v>2.1</v>
+      </c>
+      <c r="S37" s="1">
+        <f ca="1"/>
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="T37" s="1">
         <f ca="1"/>
         <v>-0.1</v>
       </c>
-      <c r="K37" s="1">
-        <f ca="1"/>
-        <v>-1.6</v>
-      </c>
-      <c r="L37" s="1">
-        <f ca="1"/>
-        <v>2</v>
-      </c>
-      <c r="M37" s="1">
-        <f ca="1"/>
-        <v>1.1100000000000001</v>
-      </c>
-      <c r="N37" s="1">
-        <f ca="1"/>
-        <v>-0.14000000000000001</v>
-      </c>
-      <c r="O37" s="1">
-        <f ca="1"/>
-        <v>0.15000000000000011</v>
-      </c>
-      <c r="P37" s="1">
-        <f ca="1"/>
-        <v>-1.08</v>
-      </c>
-      <c r="Q37" s="1">
-        <f ca="1"/>
-        <v>-2</v>
-      </c>
-      <c r="R37" s="1">
-        <f ca="1"/>
-        <v>1.05</v>
-      </c>
-      <c r="S37" s="1">
-        <f ca="1"/>
-        <v>1.1599999999999999</v>
-      </c>
-      <c r="T37" s="1">
-        <f ca="1"/>
-        <v>-1.18</v>
-      </c>
       <c r="U37" s="1">
         <f ca="1"/>
-        <v>-0.98999999999999988</v>
-      </c>
-    </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.35">
+        <v>-1.04</v>
+      </c>
+    </row>
+    <row r="38" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>10</v>
       </c>
       <c r="B38" s="1">
         <f ca="1"/>
+        <v>0.60000000000000009</v>
+      </c>
+      <c r="C38" s="1">
+        <f ca="1"/>
+        <v>0.7</v>
+      </c>
+      <c r="D38" s="1">
+        <f ca="1"/>
+        <v>0.2</v>
+      </c>
+      <c r="E38" s="1">
+        <f ca="1"/>
+        <v>0.40000000000000008</v>
+      </c>
+      <c r="F38" s="1">
+        <f ca="1"/>
+        <v>-1.4</v>
+      </c>
+      <c r="G38" s="1">
+        <f ca="1"/>
+        <v>-1.2</v>
+      </c>
+      <c r="H38" s="1">
+        <f ca="1"/>
+        <v>0.9</v>
+      </c>
+      <c r="I38" s="1">
+        <f ca="1"/>
         <v>1.4</v>
       </c>
-      <c r="C38" s="1">
-        <f ca="1"/>
-        <v>0.7</v>
-      </c>
-      <c r="D38" s="1">
-        <f ca="1"/>
-        <v>0.59999999999999987</v>
-      </c>
-      <c r="E38" s="1">
-        <f ca="1"/>
-        <v>-0.5</v>
-      </c>
-      <c r="F38" s="1">
-        <f ca="1"/>
-        <v>-1.8</v>
-      </c>
-      <c r="G38" s="1">
-        <f ca="1"/>
-        <v>-1.5</v>
-      </c>
-      <c r="H38" s="1">
-        <f ca="1"/>
-        <v>2.1</v>
-      </c>
-      <c r="I38" s="1">
-        <f ca="1"/>
-        <v>0.7</v>
-      </c>
       <c r="J38" s="1">
         <f ca="1"/>
-        <v>-1.1000000000000001</v>
+        <v>-0.70000000000000007</v>
       </c>
       <c r="K38" s="1">
         <f ca="1"/>
-        <v>-1.2</v>
+        <v>-1.4</v>
       </c>
       <c r="L38" s="1">
         <f ca="1"/>
-        <v>0.93</v>
+        <v>2</v>
       </c>
       <c r="M38" s="1">
         <f ca="1"/>
-        <v>1.0900000000000001</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="N38" s="1">
         <f ca="1"/>
-        <v>-7.999999999999996E-2</v>
+        <v>-8.9999999999999969E-2</v>
       </c>
       <c r="O38" s="1">
         <f ca="1"/>
@@ -2881,15 +2881,15 @@
       </c>
       <c r="P38" s="1">
         <f ca="1"/>
-        <v>-1.0900000000000001</v>
+        <v>-1.06</v>
       </c>
       <c r="Q38" s="1">
         <f ca="1"/>
-        <v>-0.92999999999999994</v>
+        <v>-0.86999999999999988</v>
       </c>
       <c r="R38" s="1">
         <f ca="1"/>
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="S38" s="1">
         <f ca="1"/>
@@ -2897,56 +2897,56 @@
       </c>
       <c r="T38" s="1">
         <f ca="1"/>
-        <v>-1.1499999999999999</v>
+        <v>-1.1599999999999999</v>
       </c>
       <c r="U38" s="1">
         <f ca="1"/>
-        <v>-1.02</v>
-      </c>
-    </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.35">
+        <v>-0.94999999999999984</v>
+      </c>
+    </row>
+    <row r="39" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>11</v>
       </c>
       <c r="B39" s="1">
         <f ca="1"/>
-        <v>0.8</v>
+        <v>1.8</v>
       </c>
       <c r="C39" s="1">
         <f ca="1"/>
+        <v>0.89999999999999991</v>
+      </c>
+      <c r="D39" s="1">
+        <f ca="1"/>
+        <v>-0.2</v>
+      </c>
+      <c r="E39" s="1">
+        <f ca="1"/>
+        <v>0.3</v>
+      </c>
+      <c r="F39" s="1">
+        <f ca="1"/>
+        <v>-1.6</v>
+      </c>
+      <c r="G39" s="1">
+        <f ca="1"/>
+        <v>-1.3</v>
+      </c>
+      <c r="H39" s="1">
+        <f ca="1"/>
+        <v>2.1</v>
+      </c>
+      <c r="I39" s="1">
+        <f ca="1"/>
         <v>0.6</v>
       </c>
-      <c r="D39" s="1">
-        <f ca="1"/>
-        <v>0.99999999999999978</v>
-      </c>
-      <c r="E39" s="1">
-        <f ca="1"/>
-        <v>-0.4</v>
-      </c>
-      <c r="F39" s="1">
-        <f ca="1"/>
-        <v>-1.2</v>
-      </c>
-      <c r="G39" s="1">
-        <f ca="1"/>
-        <v>-0.49999999999999978</v>
-      </c>
-      <c r="H39" s="1">
-        <f ca="1"/>
-        <v>1.3</v>
-      </c>
-      <c r="I39" s="1">
-        <f ca="1"/>
-        <v>1.3</v>
-      </c>
       <c r="J39" s="1">
         <f ca="1"/>
-        <v>-1.7</v>
+        <v>-1.9</v>
       </c>
       <c r="K39" s="1">
         <f ca="1"/>
-        <v>-0.9</v>
+        <v>-0.69999999999999984</v>
       </c>
       <c r="L39" s="1">
         <f ca="1"/>
@@ -2954,11 +2954,11 @@
       </c>
       <c r="M39" s="1">
         <f ca="1"/>
-        <v>0</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="N39" s="1">
         <f ca="1"/>
-        <v>-5.9999999999999942E-2</v>
+        <v>-6.9999999999999951E-2</v>
       </c>
       <c r="O39" s="1">
         <f ca="1"/>
@@ -2970,11 +2970,11 @@
       </c>
       <c r="Q39" s="1">
         <f ca="1"/>
-        <v>-0.91999999999999993</v>
+        <v>-0.92999999999999994</v>
       </c>
       <c r="R39" s="1">
         <f ca="1"/>
-        <v>0.99</v>
+        <v>1.04</v>
       </c>
       <c r="S39" s="1">
         <f ca="1"/>
@@ -2982,20 +2982,20 @@
       </c>
       <c r="T39" s="1">
         <f ca="1"/>
-        <v>-1.19</v>
+        <v>-1.24</v>
       </c>
       <c r="U39" s="1">
         <f ca="1"/>
-        <v>-0.97999999999999987</v>
-      </c>
-    </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.35">
+        <v>-1.02</v>
+      </c>
+    </row>
+    <row r="41" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>10</v>
       </c>
       <c r="B41" s="1">
         <f t="shared" ref="B41:U41" ca="1" si="6">AVERAGE(B29:B39)</f>
-        <v>1.0000000000000002</v>
+        <v>1</v>
       </c>
       <c r="C41" s="1">
         <f t="shared" ca="1" si="6"/>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="D41" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>0</v>
+        <v>-4.0371746350005693E-17</v>
       </c>
       <c r="E41" s="1">
         <f t="shared" ca="1" si="6"/>
@@ -3015,11 +3015,11 @@
       </c>
       <c r="G41" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>-1</v>
+        <v>-0.99999999999999989</v>
       </c>
       <c r="H41" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>1.0999999999999999</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="I41" s="1">
         <f t="shared" ca="1" si="6"/>
@@ -3039,7 +3039,7 @@
       </c>
       <c r="M41" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>0.99999999999999989</v>
+        <v>1</v>
       </c>
       <c r="N41" s="1">
         <f t="shared" ca="1" si="6"/>
@@ -3047,7 +3047,7 @@
       </c>
       <c r="O41" s="1">
         <f t="shared" ca="1" si="6"/>
-        <v>7.5697024406260668E-17</v>
+        <v>7.8220258553136033E-17</v>
       </c>
       <c r="P41" s="1">
         <f t="shared" ca="1" si="6"/>
@@ -3074,17 +3074,17 @@
         <v>-1.0999999999999999</v>
       </c>
     </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B42" s="4">
         <f t="shared" ref="B42:U42" ca="1" si="7">_xlfn.STDEV.P(B29:B39)</f>
-        <v>0.63245553203367544</v>
+        <v>0.63245553203367588</v>
       </c>
       <c r="C42" s="4">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31622776601683805</v>
+        <v>0.31622776601683877</v>
       </c>
       <c r="D42" s="4">
         <f t="shared" ca="1" si="7"/>
@@ -3096,19 +3096,19 @@
       </c>
       <c r="F42" s="4">
         <f t="shared" ca="1" si="7"/>
-        <v>0.6324555320336761</v>
+        <v>0.63245553203367588</v>
       </c>
       <c r="G42" s="4">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31622776601683783</v>
+        <v>0.31622776601683844</v>
       </c>
       <c r="H42" s="4">
         <f t="shared" ca="1" si="7"/>
-        <v>0.63245553203367588</v>
+        <v>0.63245553203367566</v>
       </c>
       <c r="I42" s="4">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31622776601683822</v>
+        <v>0.31622776601683783</v>
       </c>
       <c r="J42" s="4">
         <f t="shared" ca="1" si="7"/>
@@ -3116,7 +3116,7 @@
       </c>
       <c r="K42" s="4">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31622776601683822</v>
+        <v>0.31622776601683783</v>
       </c>
       <c r="L42" s="1">
         <f t="shared" ca="1" si="7"/>
@@ -3124,7 +3124,7 @@
       </c>
       <c r="M42" s="1">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31780497164141469</v>
+        <v>0.31780497164141414</v>
       </c>
       <c r="N42" s="1">
         <f t="shared" ca="1" si="7"/>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="P42" s="1">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31780497164141358</v>
+        <v>0.31780497164141319</v>
       </c>
       <c r="Q42" s="1">
         <f t="shared" ca="1" si="7"/>
@@ -3144,7 +3144,7 @@
       </c>
       <c r="R42" s="1">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31780497164141336</v>
+        <v>0.31780497164141375</v>
       </c>
       <c r="S42" s="1">
         <f t="shared" ca="1" si="7"/>
@@ -3152,64 +3152,64 @@
       </c>
       <c r="T42" s="1">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31780497164141414</v>
+        <v>0.31780497164141375</v>
       </c>
       <c r="U42" s="1">
         <f t="shared" ca="1" si="7"/>
-        <v>0.31780497164141414</v>
-      </c>
-    </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.35">
+        <v>0.31780497164141486</v>
+      </c>
+    </row>
+    <row r="43" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>12</v>
       </c>
       <c r="B43" s="1">
         <f t="shared" ref="B43:U43" ca="1" si="8">_xlfn.SKEW.P(B29:B39)</f>
-        <v>-1.0389416599759277E-15</v>
+        <v>4.0371746350005693E-17</v>
       </c>
       <c r="C43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>7.2669143430010251E-16</v>
+        <v>8.1878948066105295E-16</v>
       </c>
       <c r="D43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>-5.2483270255007403E-16</v>
+        <v>-4.0056342081646272E-16</v>
       </c>
       <c r="E43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>4.8446095620006827E-16</v>
+        <v>4.6427508302506544E-16</v>
       </c>
       <c r="F43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>-2.7124767078910076E-16</v>
+        <v>-2.8260222445003984E-16</v>
       </c>
       <c r="G43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>7.6706318065010816E-16</v>
+        <v>-2.6241635127503701E-16</v>
       </c>
       <c r="H43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>6.4531713306337224E-16</v>
+        <v>-3.6334571715005125E-16</v>
       </c>
       <c r="I43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>1.1304088978001594E-15</v>
+        <v>1.2515241368501765E-15</v>
       </c>
       <c r="J43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>-7.5697024406260675E-16</v>
+        <v>-8.0743492700011382E-16</v>
       </c>
       <c r="K43" s="1">
         <f t="shared" ca="1" si="8"/>
-        <v>-6.7118028306884468E-16</v>
+        <v>-5.2483270255007403E-16</v>
       </c>
       <c r="L43" s="4">
         <f t="shared" ca="1" si="8"/>
-        <v>2.7945403348921536</v>
+        <v>2.7945403348921523</v>
       </c>
       <c r="M43" s="4">
         <f t="shared" ca="1" si="8"/>
-        <v>-2.7945403348921505</v>
+        <v>-2.7945403348921536</v>
       </c>
       <c r="N43" s="4">
         <f t="shared" ca="1" si="8"/>
@@ -3229,22 +3229,22 @@
       </c>
       <c r="R43" s="4">
         <f t="shared" ca="1" si="8"/>
-        <v>2.7945403348921518</v>
+        <v>2.7945403348921514</v>
       </c>
       <c r="S43" s="4">
         <f t="shared" ca="1" si="8"/>
-        <v>-2.7945403348921518</v>
+        <v>-2.7945403348921505</v>
       </c>
       <c r="T43" s="4">
         <f t="shared" ca="1" si="8"/>
-        <v>2.7945403348921518</v>
+        <v>2.79454033489215</v>
       </c>
       <c r="U43" s="4">
         <f t="shared" ca="1" si="8"/>
-        <v>-2.794540334892154</v>
-      </c>
-    </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.35">
+        <v>-2.7945403348921518</v>
+      </c>
+    </row>
+    <row r="44" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>13</v>
       </c>
@@ -3254,15 +3254,15 @@
       </c>
       <c r="C44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>-1.2000000000000015</v>
+        <v>-1.2000000000000002</v>
       </c>
       <c r="D44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>-1.1999999999999997</v>
+        <v>-1.2000000000000002</v>
       </c>
       <c r="E44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>-1.1999999999999997</v>
+        <v>-1.200000000000002</v>
       </c>
       <c r="F44" s="1">
         <f t="shared" ca="1" si="9"/>
@@ -3274,11 +3274,11 @@
       </c>
       <c r="H44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>-1.2000000000000002</v>
+        <v>-1.1999999999999997</v>
       </c>
       <c r="I44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>-1.2000000000000002</v>
+        <v>-1.2000000000000011</v>
       </c>
       <c r="J44" s="1">
         <f t="shared" ca="1" si="9"/>
@@ -3290,11 +3290,11 @@
       </c>
       <c r="L44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993702</v>
+        <v>10.711250530993684</v>
       </c>
       <c r="M44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993684</v>
+        <v>10.711250530993706</v>
       </c>
       <c r="N44" s="1">
         <f t="shared" ca="1" si="9"/>
@@ -3302,7 +3302,7 @@
       </c>
       <c r="O44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993688</v>
+        <v>10.711250530993684</v>
       </c>
       <c r="P44" s="1">
         <f t="shared" ca="1" si="9"/>
@@ -3310,26 +3310,26 @@
       </c>
       <c r="Q44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993702</v>
+        <v>10.711250530993706</v>
       </c>
       <c r="R44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993688</v>
+        <v>10.711250530993684</v>
       </c>
       <c r="S44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993695</v>
+        <v>10.711250530993688</v>
       </c>
       <c r="T44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993691</v>
+        <v>10.711250530993684</v>
       </c>
       <c r="U44" s="1">
         <f t="shared" ca="1" si="9"/>
-        <v>10.711250530993706</v>
-      </c>
-    </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.35">
+        <v>10.711250530993691</v>
+      </c>
+    </row>
+    <row r="45" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>14</v>
       </c>
@@ -3414,7 +3414,7 @@
         <v>-2.1</v>
       </c>
     </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>15</v>
       </c>
@@ -3499,62 +3499,62 @@
         <v>-0.94999999999999984</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>16</v>
       </c>
       <c r="B47" s="1">
         <f ca="1">CORREL(B29:B39,C29:C39)</f>
-        <v>-0.21818181818181812</v>
+        <v>-0.10000000000000006</v>
       </c>
       <c r="D47" s="1">
         <f ca="1">CORREL(D29:D39,E29:E39)</f>
-        <v>-0.30909090909090897</v>
+        <v>-0.35454545454545439</v>
       </c>
       <c r="F47" s="1">
         <f ca="1">CORREL(F29:F39,G29:G39)</f>
-        <v>6.3636363636363588E-2</v>
+        <v>0.31818181818181807</v>
       </c>
       <c r="H47" s="1">
         <f ca="1">CORREL(H29:H39,I29:I39)</f>
-        <v>6.3636363636363519E-2</v>
+        <v>0.11818181818181828</v>
       </c>
       <c r="J47" s="1">
         <f ca="1">CORREL(J29:J39,K29:K39)</f>
-        <v>-0.28181818181818186</v>
+        <v>-0.3545454545454545</v>
       </c>
       <c r="L47" s="1">
         <f ca="1">CORREL(L29:L39,M29:M39)</f>
-        <v>0.10126012601260134</v>
+        <v>6.4356435643564386E-2</v>
       </c>
       <c r="N47" s="1">
         <f ca="1">CORREL(N29:N39,O29:O39)</f>
-        <v>0.10513051305130515</v>
+        <v>9.0009000900090022E-2</v>
       </c>
       <c r="P47" s="1">
         <f ca="1">CORREL(P29:P39,Q29:Q39)</f>
-        <v>0.1245724572457247</v>
+        <v>0.12934293429342944</v>
       </c>
       <c r="R47" s="1">
         <f ca="1">CORREL(R29:R39,S29:S39)</f>
-        <v>0.12763276327632767</v>
+        <v>3.8703870387038646E-2</v>
       </c>
       <c r="T47" s="1">
         <f ca="1">CORREL(T29:T39,U29:U39)</f>
-        <v>2.1062106210620948E-2</v>
-      </c>
-    </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.35">
+        <v>1.3861386138613749E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>17</v>
       </c>
       <c r="B48">
         <f t="array" aca="1" ref="B48" ca="1">SUMPRODUCT((B29:B39&gt;C29:C39)*1)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C48">
         <f t="array" aca="1" ref="C48" ca="1">SUMPRODUCT((B29:B39&lt;C29:C39)*1)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D48">
         <f t="array" aca="1" ref="D48" ca="1">SUMPRODUCT((D29:D39&gt;E29:E39)*1)</f>
@@ -3574,19 +3574,19 @@
       </c>
       <c r="H48">
         <f t="array" aca="1" ref="H48" ca="1">SUMPRODUCT((H29:H39&gt;I29:I39)*1)</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I48">
         <f t="array" aca="1" ref="I48" ca="1">SUMPRODUCT((H29:H39&lt;I29:I39)*1)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J48">
         <f t="array" aca="1" ref="J48" ca="1">SUMPRODUCT((J29:J39&gt;K29:K39)*1)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K48">
         <f t="array" aca="1" ref="K48" ca="1">SUMPRODUCT((J29:J39&lt;K29:K39)*1)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L48">
         <f t="array" aca="1" ref="L48" ca="1">SUMPRODUCT((L29:L39&gt;M29:M39)*1)</f>
@@ -3629,7 +3629,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A49" s="5" t="s">
         <v>18</v>
       </c>
@@ -3647,11 +3647,11 @@
       </c>
       <c r="H49" s="6" t="str">
         <f ca="1">IF(H48&gt;I48,"A",IF(I48&gt;H48,"B","Equal"))</f>
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="J49" s="6" t="str">
         <f ca="1">IF(J48&gt;K48,"A",IF(K48&gt;J48,"B","Equal"))</f>
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="L49" s="6" t="str">
         <f ca="1">IF(L48&gt;M48,"A",IF(M48&gt;L48,"B","Equal"))</f>
@@ -3674,13 +3674,13 @@
         <v>B</v>
       </c>
     </row>
-    <row r="50" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>19</v>
       </c>
       <c r="B50">
         <f ca="1">MAX(B48:C48)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D50">
         <f ca="1">MAX(D48:E48)</f>
@@ -3719,12 +3719,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="54" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A54" s="2"/>
       <c r="B54" s="11" t="s">
         <v>0</v>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="U54" s="12"/>
     </row>
-    <row r="55" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B55" s="1">
         <v>0</v>
       </c>
@@ -3835,7 +3835,7 @@
       <c r="Z55" s="1"/>
       <c r="AB55" s="1"/>
     </row>
-    <row r="56" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B56" s="1">
         <v>0.2</v>
       </c>
@@ -3903,7 +3903,7 @@
       <c r="Z56" s="1"/>
       <c r="AB56" s="1"/>
     </row>
-    <row r="57" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B57" s="1">
         <v>0.4</v>
       </c>
@@ -3971,7 +3971,7 @@
       <c r="Z57" s="1"/>
       <c r="AB57" s="1"/>
     </row>
-    <row r="58" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B58" s="1">
         <v>0.60000000000000009</v>
       </c>
@@ -4039,7 +4039,7 @@
       <c r="Z58" s="1"/>
       <c r="AB58" s="1"/>
     </row>
-    <row r="59" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B59" s="1">
         <v>0.8</v>
       </c>
@@ -4107,7 +4107,7 @@
       <c r="Z59" s="1"/>
       <c r="AB59" s="1"/>
     </row>
-    <row r="60" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B60" s="1">
         <v>1</v>
       </c>
@@ -4175,7 +4175,7 @@
       <c r="Z60" s="1"/>
       <c r="AB60" s="1"/>
     </row>
-    <row r="61" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B61" s="1">
         <v>1.2</v>
       </c>
@@ -4243,7 +4243,7 @@
       <c r="Z61" s="1"/>
       <c r="AB61" s="1"/>
     </row>
-    <row r="62" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B62" s="1">
         <v>1.4</v>
       </c>
@@ -4311,7 +4311,7 @@
       <c r="Z62" s="1"/>
       <c r="AB62" s="1"/>
     </row>
-    <row r="63" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B63" s="1">
         <v>1.6</v>
       </c>
@@ -4379,7 +4379,7 @@
       <c r="Z63" s="1"/>
       <c r="AB63" s="1"/>
     </row>
-    <row r="64" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B64" s="1">
         <v>1.8</v>
       </c>
@@ -4447,7 +4447,7 @@
       <c r="Z64" s="1"/>
       <c r="AB64" s="1"/>
     </row>
-    <row r="65" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B65" s="1">
         <v>2</v>
       </c>
@@ -4515,7 +4515,7 @@
       <c r="Z65" s="1"/>
       <c r="AB65" s="1"/>
     </row>
-    <row r="67" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>10</v>
       </c>
@@ -4604,7 +4604,7 @@
       <c r="Y67" s="1"/>
       <c r="Z67" s="1"/>
     </row>
-    <row r="68" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
         <v>11</v>
       </c>
@@ -4693,7 +4693,7 @@
       <c r="Y68" s="1"/>
       <c r="Z68" s="1"/>
     </row>
-    <row r="69" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>12</v>
       </c>
@@ -4782,7 +4782,7 @@
       <c r="Y69" s="1"/>
       <c r="Z69" s="1"/>
     </row>
-    <row r="70" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>13</v>
       </c>
@@ -4871,7 +4871,7 @@
       <c r="Y70" s="1"/>
       <c r="Z70" s="1"/>
     </row>
-    <row r="71" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>14</v>
       </c>
@@ -4960,7 +4960,7 @@
       <c r="Y71" s="1"/>
       <c r="Z71" s="1"/>
     </row>
-    <row r="72" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>15</v>
       </c>
@@ -5049,7 +5049,7 @@
       <c r="Y72" s="1"/>
       <c r="Z72" s="1"/>
     </row>
-    <row r="73" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>16</v>
       </c>
@@ -5096,7 +5096,7 @@
       <c r="W73" s="1"/>
       <c r="Y73" s="1"/>
     </row>
-    <row r="74" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="s">
         <v>17</v>
       </c>
@@ -5181,7 +5181,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="75" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A75" s="5" t="s">
         <v>18</v>
       </c>
@@ -5228,7 +5228,7 @@
       <c r="W75" s="6"/>
       <c r="Y75" s="6"/>
     </row>
-    <row r="76" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>19</v>
       </c>
@@ -5273,12 +5273,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="78" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A78" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="80" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A80" s="2"/>
       <c r="B80" s="11" t="s">
         <v>0</v>
@@ -5321,7 +5321,7 @@
       </c>
       <c r="U80" s="12"/>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B81" s="1">
         <v>0.60000000000000009</v>
       </c>
@@ -5384,7 +5384,7 @@
       </c>
       <c r="V81" s="1"/>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B82" s="1">
         <v>0.8</v>
       </c>
@@ -5447,7 +5447,7 @@
       </c>
       <c r="V82" s="1"/>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B83" s="1">
         <v>1</v>
       </c>
@@ -5510,7 +5510,7 @@
       </c>
       <c r="V83" s="1"/>
     </row>
-    <row r="84" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B84" s="1">
         <v>1.2</v>
       </c>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="V84" s="1"/>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B85" s="1">
         <v>1.4</v>
       </c>
@@ -5636,7 +5636,7 @@
       </c>
       <c r="V85" s="1"/>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B86" s="1">
         <v>1.6</v>
       </c>
@@ -5699,7 +5699,7 @@
       </c>
       <c r="V86" s="1"/>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B87" s="1">
         <v>1.8</v>
       </c>
@@ -5762,7 +5762,7 @@
       </c>
       <c r="V87" s="1"/>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B88" s="1">
         <v>2</v>
       </c>
@@ -5825,7 +5825,7 @@
       </c>
       <c r="V88" s="1"/>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B89" s="1">
         <v>0</v>
       </c>
@@ -5888,7 +5888,7 @@
       </c>
       <c r="V89" s="1"/>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B90" s="1">
         <v>0.2</v>
       </c>
@@ -5951,7 +5951,7 @@
       </c>
       <c r="V90" s="1"/>
     </row>
-    <row r="91" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B91" s="1">
         <v>0.4</v>
       </c>
@@ -6014,7 +6014,7 @@
       </c>
       <c r="V91" s="1"/>
     </row>
-    <row r="93" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>10</v>
       </c>
@@ -6099,7 +6099,7 @@
         <v>-1.0999999999999999</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A94" s="3" t="s">
         <v>11</v>
       </c>
@@ -6184,7 +6184,7 @@
         <v>0.31780497164141375</v>
       </c>
     </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>12</v>
       </c>
@@ -6269,7 +6269,7 @@
         <v>-2.794540334892154</v>
       </c>
     </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>13</v>
       </c>
@@ -6354,7 +6354,7 @@
         <v>10.711250530993706</v>
       </c>
     </row>
-    <row r="97" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>14</v>
       </c>
@@ -6439,7 +6439,7 @@
         <v>-2.1</v>
       </c>
     </row>
-    <row r="98" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>15</v>
       </c>
@@ -6524,7 +6524,7 @@
         <v>-0.94999999999999984</v>
       </c>
     </row>
-    <row r="99" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>16</v>
       </c>
@@ -6569,7 +6569,7 @@
         <v>0.20513051305130531</v>
       </c>
     </row>
-    <row r="100" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A100" s="3" t="s">
         <v>17</v>
       </c>
@@ -6654,7 +6654,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="101" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A101" s="5" t="s">
         <v>18</v>
       </c>
@@ -6699,7 +6699,7 @@
         <v>B</v>
       </c>
     </row>
-    <row r="102" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>19</v>
       </c>
@@ -6744,15 +6744,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="104" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A104" s="8" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="105" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A105" s="8"/>
     </row>
-    <row r="106" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B106" s="8" t="s">
         <v>0</v>
       </c>
@@ -6784,7 +6784,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="107" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A107" s="9" t="s">
         <v>24</v>
       </c>
@@ -6819,77 +6819,77 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="108" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A108" s="9" t="s">
         <v>25</v>
       </c>
       <c r="B108" s="10">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="D108" s="10">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="F108" s="10">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H108" s="10">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="J108" s="10">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="L108" s="10">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="N108" s="10">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="P108" s="10">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="R108" s="10">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="T108" s="10">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="109" spans="1:21" x14ac:dyDescent="0.35">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="109" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A109" s="9" t="s">
         <v>26</v>
       </c>
       <c r="B109" s="10">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="D109" s="10">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="F109" s="10">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="H109" s="10">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="J109" s="10">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="L109" s="10">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="N109" s="10">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="P109" s="10">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="R109" s="10">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="T109" s="10">
-        <v>1.4</v>
-      </c>
-    </row>
-    <row r="110" spans="1:21" x14ac:dyDescent="0.35">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="110" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A110" s="9" t="s">
         <v>27</v>
       </c>
@@ -6926,18 +6926,21 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="T28:U28"/>
-    <mergeCell ref="N80:O80"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="P54:Q54"/>
-    <mergeCell ref="T54:U54"/>
-    <mergeCell ref="F80:G80"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="J80:K80"/>
-    <mergeCell ref="P80:Q80"/>
-    <mergeCell ref="R80:S80"/>
-    <mergeCell ref="T80:U80"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="L80:M80"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="F54:G54"/>
+    <mergeCell ref="H54:I54"/>
+    <mergeCell ref="N54:O54"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="P28:Q28"/>
+    <mergeCell ref="H28:I28"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="T2:U2"/>
@@ -6948,24 +6951,21 @@
     <mergeCell ref="F28:G28"/>
     <mergeCell ref="R28:S28"/>
     <mergeCell ref="J28:K28"/>
+    <mergeCell ref="L28:M28"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="J80:K80"/>
+    <mergeCell ref="P80:Q80"/>
+    <mergeCell ref="R80:S80"/>
+    <mergeCell ref="T28:U28"/>
+    <mergeCell ref="N80:O80"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="P54:Q54"/>
+    <mergeCell ref="T54:U54"/>
+    <mergeCell ref="F80:G80"/>
+    <mergeCell ref="T80:U80"/>
     <mergeCell ref="D80:E80"/>
-    <mergeCell ref="L28:M28"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="P28:Q28"/>
-    <mergeCell ref="H28:I28"/>
     <mergeCell ref="H80:I80"/>
-    <mergeCell ref="B80:C80"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="R2:S2"/>
-    <mergeCell ref="L80:M80"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="F54:G54"/>
-    <mergeCell ref="H54:I54"/>
-    <mergeCell ref="N54:O54"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6974,9 +6974,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:K21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B2" s="11" t="s">
         <v>0</v>
       </c>
@@ -6998,7 +6998,7 @@
       </c>
       <c r="K2" s="12"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B3" s="1">
         <v>0</v>
       </c>
@@ -7038,7 +7038,7 @@
         <v>-1.6</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B4" s="1">
         <v>0.2</v>
       </c>
@@ -7078,7 +7078,7 @@
         <v>-1.5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B5" s="1">
         <v>0.4</v>
       </c>
@@ -7118,7 +7118,7 @@
         <v>-1.4000000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B6" s="1">
         <v>0.60000000000000009</v>
       </c>
@@ -7158,7 +7158,7 @@
         <v>-1.3000000000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B7" s="1">
         <v>0.8</v>
       </c>
@@ -7198,7 +7198,7 @@
         <v>-1.2000000000000002</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B8" s="1">
         <v>1</v>
       </c>
@@ -7238,7 +7238,7 @@
         <v>-1.1000000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B9" s="1">
         <v>1.2</v>
       </c>
@@ -7278,7 +7278,7 @@
         <v>-0.99999999999999989</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B10" s="1">
         <v>1.4</v>
       </c>
@@ -7318,7 +7318,7 @@
         <v>-0.9</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B11" s="1">
         <v>1.6</v>
       </c>
@@ -7358,7 +7358,7 @@
         <v>-0.79999999999999993</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B12" s="1">
         <v>1.8</v>
       </c>
@@ -7398,7 +7398,7 @@
         <v>-0.70000000000000007</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B13" s="1">
         <v>2</v>
       </c>
@@ -7438,7 +7438,7 @@
         <v>-0.6</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -7483,7 +7483,7 @@
         <v>-1.1000000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>11</v>
       </c>
@@ -7528,7 +7528,7 @@
         <v>0.31622776601683822</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -7573,7 +7573,7 @@
         <v>5.2483270255007403E-16</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -7618,7 +7618,7 @@
         <v>-1.2000000000000011</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>14</v>
       </c>
@@ -7663,7 +7663,7 @@
         <v>-1.6</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>15</v>
       </c>
@@ -7708,7 +7708,7 @@
         <v>-0.6</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -7748,9 +7748,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A2:K21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B2" s="11" t="s">
         <v>5</v>
       </c>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="K2" s="12"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B3" s="1">
         <v>0.85</v>
       </c>
@@ -7812,7 +7812,7 @@
         <v>-1.05</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B4" s="1">
         <v>0.86</v>
       </c>
@@ -7852,7 +7852,7 @@
         <v>-1.04</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B5" s="1">
         <v>0.87</v>
       </c>
@@ -7892,7 +7892,7 @@
         <v>-1.03</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B6" s="1">
         <v>0.88</v>
       </c>
@@ -7932,7 +7932,7 @@
         <v>-1.02</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B7" s="1">
         <v>0.89</v>
       </c>
@@ -7972,7 +7972,7 @@
         <v>-1.01</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B8" s="1">
         <v>0.91</v>
       </c>
@@ -8012,7 +8012,7 @@
         <v>-0.98999999999999988</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B9" s="1">
         <v>0.92</v>
       </c>
@@ -8052,7 +8052,7 @@
         <v>-0.97999999999999987</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B10" s="1">
         <v>0.93</v>
       </c>
@@ -8092,7 +8092,7 @@
         <v>-0.97000000000000008</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B11" s="1">
         <v>0.94000000000000006</v>
       </c>
@@ -8132,7 +8132,7 @@
         <v>-0.96000000000000008</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B12" s="1">
         <v>0.95000000000000007</v>
       </c>
@@ -8172,7 +8172,7 @@
         <v>-0.95000000000000007</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B13" s="1">
         <v>2</v>
       </c>
@@ -8212,7 +8212,7 @@
         <v>-2.1</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -8257,7 +8257,7 @@
         <v>-1.0999999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -8302,7 +8302,7 @@
         <v>0.31780497164141414</v>
       </c>
     </row>
-    <row r="17" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>12</v>
       </c>
@@ -8347,7 +8347,7 @@
         <v>-2.7945403348921536</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -8392,7 +8392,7 @@
         <v>10.711250530993702</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>14</v>
       </c>
@@ -8437,7 +8437,7 @@
         <v>-2.1</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>15</v>
       </c>
@@ -8482,7 +8482,7 @@
         <v>-0.95000000000000007</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>16</v>
       </c>

</xml_diff>